<commit_message>
Add 20k-iteration GradInversion results on driver-split model: S2_full (DINOv2) and S1_full (no teacher), plots and Excel
</commit_message>
<xml_diff>
--- a/fedkd_gia/results/fedkd_gia_results.xlsx
+++ b/fedkd_gia/results/fedkd_gia_results.xlsx
@@ -7,10 +7,17 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Baseline_Rounds" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Baseline_Clients" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Baseline_HeldOut" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Baseline_Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="GI_Comparison" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Baseline_Rounds" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Baseline_Clients" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Baseline_HeldOut" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Baseline_Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="S1_full" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="S1_full_Images" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="S2_full" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="S2_full_Images" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="S1_full_Plots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="S2_full_Plots" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,9 +26,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -68,17 +76,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -153,6 +164,426 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>75</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>99</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>123</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>75</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>99</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>123</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4819650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4276725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4819650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4276725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -444,6 +875,381 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>none_20k: PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>none_20k: gain over floor (dB)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>none_20k: PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>dinov2_20k: PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>dinov2_20k: gain over floor (dB)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>dinov2_20k: PSNR best seed (dB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>p002</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>9.40250867502931</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>10.18981834941837</v>
+      </c>
+      <c r="D2" s="3">
+        <f>C2-$B2</f>
+        <v/>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>10.02273675431274</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>11.95569679194365</v>
+      </c>
+      <c r="G2" s="3">
+        <f>F2-$B2</f>
+        <v/>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>11.9642847229547</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>9.988775402453584</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>10.92384761775596</v>
+      </c>
+      <c r="D3" s="3">
+        <f>C3-$B3</f>
+        <v/>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>10.76693620718362</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>12.01081569052551</v>
+      </c>
+      <c r="G3" s="3">
+        <f>F3-$B3</f>
+        <v/>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>11.82164962106386</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>10.14880432187795</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>10.65960550177276</v>
+      </c>
+      <c r="D4" s="3">
+        <f>C4-$B4</f>
+        <v/>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>10.35919985618149</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>10.47159694146267</v>
+      </c>
+      <c r="G4" s="3">
+        <f>F4-$B4</f>
+        <v/>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>10.33662003823281</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>10.07038371983996</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>9.879232901906896</v>
+      </c>
+      <c r="D5" s="3">
+        <f>C5-$B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>9.619753613356174</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>12.00279410983525</v>
+      </c>
+      <c r="G5" s="3">
+        <f>F5-$B5</f>
+        <v/>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>11.54788435056746</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>p021</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>9.450420919396539</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>10.15026036519444</v>
+      </c>
+      <c r="D6" s="3">
+        <f>C6-$B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>9.839114019807274</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>10.27059412332502</v>
+      </c>
+      <c r="G6" s="3">
+        <f>F6-$B6</f>
+        <v/>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>10.04729325639967</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>9.082354949847025</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>9.769899243281543</v>
+      </c>
+      <c r="D7" s="3">
+        <f>C7-$B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>9.753765040360975</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>9.597271589453804</v>
+      </c>
+      <c r="G7" s="3">
+        <f>F7-$B7</f>
+        <v/>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>9.647701764458878</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mean</t>
+        </is>
+      </c>
+      <c r="B8" s="5">
+        <f>AVERAGE(B2:B7)</f>
+        <v/>
+      </c>
+      <c r="C8" s="5">
+        <f>AVERAGE(C2:C7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="5">
+        <f>AVERAGE(D2:D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="5">
+        <f>AVERAGE(E2:E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="5">
+        <f>AVERAGE(F2:F7)</f>
+        <v/>
+      </c>
+      <c r="G8" s="5">
+        <f>AVERAGE(G2:G7)</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>AVERAGE(H2:H7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Clients above floor</t>
+        </is>
+      </c>
+      <c r="D9" s="4">
+        <f>COUNTIF(D2:D7,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
+        <f>COUNTIF(G2:G7,"&gt;0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Settings: none_20k = S1_full no teacher, 20k iterations; dinov2_20k = S2_full DINOv2 surrogate, 20k iterations</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Gain over floor = consensus PSNR minus PSNR of a uniform gray image (no-information reference).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>All attacks: round-30 victim gradient, batch 8, 2 seeds, TV 1, no Langevin noise; 4000 iterations except the _20k columns (S1_full / S2_full: 20000 iterations, 6 clients).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_all_clients.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_vs_iteration.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_all_clients.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_vs_iteration.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -497,22 +1303,22 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="7" t="n">
         <v>0.08496221005994266</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="8" t="n">
         <v>0.01566554541086016</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="7" t="n">
         <v>0.07591824075649956</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="7" t="n">
         <v>0.146</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="9" t="n">
         <v>19.47545262177785</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="8" t="n">
         <v>0.07756841616509436</v>
       </c>
     </row>
@@ -520,22 +1326,22 @@
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="7" t="n">
         <v>0.1532447224394058</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="8" t="n">
         <v>0.1073283391177897</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="7" t="n">
         <v>0.1328554887485038</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="7" t="n">
         <v>0.1435238095238095</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="9" t="n">
         <v>19.33178738355637</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="8" t="n">
         <v>0.07503990313836767</v>
       </c>
     </row>
@@ -543,22 +1349,22 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="7" t="n">
         <v>0.1675788376335679</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="8" t="n">
         <v>0.1194070719906583</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="7" t="n">
         <v>0.1442587725644865</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="7" t="n">
         <v>0.1436190476190476</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="9" t="n">
         <v>19.32938230037689</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="8" t="n">
         <v>0.07685557329454681</v>
       </c>
     </row>
@@ -566,22 +1372,22 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="7" t="n">
         <v>0.2791243158717748</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="8" t="n">
         <v>0.262471497600986</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="7" t="n">
         <v>0.2355453046335879</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="7" t="n">
         <v>0.1375238095238095</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="9" t="n">
         <v>19.46547210613886</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="8" t="n">
         <v>0.06627256951201639</v>
       </c>
     </row>
@@ -589,22 +1395,22 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="7" t="n">
         <v>0.3145686734427938</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="8" t="n">
         <v>0.2986755298044492</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="7" t="n">
         <v>0.265826705433421</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" s="7" t="n">
         <v>0.1486190476190476</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="9" t="n">
         <v>19.64586573839188</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="8" t="n">
         <v>0.07808343888601603</v>
       </c>
     </row>
@@ -612,22 +1418,22 @@
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="7" t="n">
         <v>0.3575710190252802</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="8" t="n">
         <v>0.346946224872787</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="7" t="n">
         <v>0.3070942539307317</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="7" t="n">
         <v>0.154</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="9" t="n">
         <v>19.64620331923167</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" s="8" t="n">
         <v>0.08566612006631409</v>
       </c>
     </row>
@@ -635,22 +1441,22 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="7" t="n">
         <v>0.3588741204065676</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="8" t="n">
         <v>0.3623378867234874</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="7" t="n">
         <v>0.3075950804032495</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="7" t="n">
         <v>0.148</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="9" t="n">
         <v>19.86083125273387</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="8" t="n">
         <v>0.08327593289847908</v>
       </c>
     </row>
@@ -658,22 +1464,22 @@
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="7" t="n">
         <v>0.381808704717227</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="8" t="n">
         <v>0.379626872458671</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" s="7" t="n">
         <v>0.3306694355475639</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="7" t="n">
         <v>0.1468095238095238</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="9" t="n">
         <v>19.66802999973297</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="G9" s="8" t="n">
         <v>0.08026616184681187</v>
       </c>
     </row>
@@ -681,22 +1487,22 @@
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="7" t="n">
         <v>0.4123012770393537</v>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="8" t="n">
         <v>0.410373743207377</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="7" t="n">
         <v>0.3636706349192342</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="7" t="n">
         <v>0.1445714285714285</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="9" t="n">
         <v>19.67550832827886</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="G10" s="8" t="n">
         <v>0.07830577804481056</v>
       </c>
     </row>
@@ -704,22 +1510,22 @@
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="7" t="n">
         <v>0.4211623664321084</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="8" t="n">
         <v>0.4142323018193015</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="7" t="n">
         <v>0.3740045379048176</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="7" t="n">
         <v>0.137</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="9" t="n">
         <v>19.68845857381821</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="8" t="n">
         <v>0.06814269790844392</v>
       </c>
     </row>
@@ -727,22 +1533,22 @@
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="7" t="n">
         <v>0.4300234558248632</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="8" t="n">
         <v>0.4265767772436201</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="7" t="n">
         <v>0.3847764633708072</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="7" t="n">
         <v>0.1347619047619048</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="9" t="n">
         <v>19.70091542005539</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="G12" s="8" t="n">
         <v>0.07031936049956421</v>
       </c>
     </row>
@@ -750,22 +1556,22 @@
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="7" t="n">
         <v>0.4331508991399531</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="8" t="n">
         <v>0.4227757902418722</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="7" t="n">
         <v>0.3890370319089186</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="7" t="n">
         <v>0.1575714285714286</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="9" t="n">
         <v>19.88898579676946</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="G13" s="8" t="n">
         <v>0.08511132501339047</v>
       </c>
     </row>
@@ -773,22 +1579,22 @@
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" s="7" t="n">
         <v>0.4422726088089654</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="8" t="n">
         <v>0.4304502263741757</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="7" t="n">
         <v>0.3981567643722749</v>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E14" s="7" t="n">
         <v>0.1394285714285714</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="9" t="n">
         <v>19.74798041184743</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="G14" s="8" t="n">
         <v>0.0732813331647664</v>
       </c>
     </row>
@@ -796,22 +1602,22 @@
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" s="7" t="n">
         <v>0.4459212926765702</v>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="8" t="n">
         <v>0.4312343907355803</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="7" t="n">
         <v>0.4027306645120445</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="7" t="n">
         <v>0.140952380952381</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="9" t="n">
         <v>19.73155637582143</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="G15" s="8" t="n">
         <v>0.07942444210179009</v>
       </c>
     </row>
@@ -819,22 +1625,22 @@
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="7" t="n">
         <v>0.4628616106333073</v>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" s="8" t="n">
         <v>0.4511819257774817</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="7" t="n">
         <v>0.4178956996462162</v>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E16" s="7" t="n">
         <v>0.1425238095238095</v>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F16" s="9" t="n">
         <v>19.63770779371261</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="G16" s="8" t="n">
         <v>0.07362040799197524</v>
       </c>
     </row>
@@ -842,22 +1648,22 @@
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" s="7" t="n">
         <v>0.45426114151681</v>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="8" t="n">
         <v>0.4454771061547023</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" s="7" t="n">
         <v>0.4128420193481401</v>
       </c>
-      <c r="E17" s="3" t="n">
+      <c r="E17" s="7" t="n">
         <v>0.1332857142857143</v>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F17" s="9" t="n">
         <v>19.92192540168762</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="G17" s="8" t="n">
         <v>0.06578514619218143</v>
       </c>
     </row>
@@ -865,22 +1671,22 @@
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" s="7" t="n">
         <v>0.4448788115715402</v>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C18" s="8" t="n">
         <v>0.4282325853818291</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" s="7" t="n">
         <v>0.4038510149618315</v>
       </c>
-      <c r="E18" s="3" t="n">
+      <c r="E18" s="7" t="n">
         <v>0.1418571428571428</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" s="9" t="n">
         <v>19.88053689002991</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="G18" s="8" t="n">
         <v>0.07319832353502118</v>
       </c>
     </row>
@@ -888,22 +1694,22 @@
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" s="7" t="n">
         <v>0.4412301277039354</v>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="8" t="n">
         <v>0.4351936565302833</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" s="7" t="n">
         <v>0.4021329431167455</v>
       </c>
-      <c r="E19" s="3" t="n">
+      <c r="E19" s="7" t="n">
         <v>0.138</v>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="9" t="n">
         <v>19.81049696207047</v>
       </c>
-      <c r="G19" s="4" t="n">
+      <c r="G19" s="8" t="n">
         <v>0.0696663291427214</v>
       </c>
     </row>
@@ -911,22 +1717,22 @@
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" s="7" t="n">
         <v>0.4639040917383372</v>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C20" s="8" t="n">
         <v>0.4547669038854646</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" s="7" t="n">
         <v>0.4263194071775846</v>
       </c>
-      <c r="E20" s="3" t="n">
+      <c r="E20" s="7" t="n">
         <v>0.1434285714285715</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="9" t="n">
         <v>19.66176524559657</v>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="G20" s="8" t="n">
         <v>0.07097761222298876</v>
       </c>
     </row>
@@ -934,22 +1740,22 @@
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="7" t="n">
         <v>0.4472243940578577</v>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="8" t="n">
         <v>0.4355490874286445</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" s="7" t="n">
         <v>0.4064658432489119</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="E21" s="7" t="n">
         <v>0.1325238095238095</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="9" t="n">
         <v>19.92225342988968</v>
       </c>
-      <c r="G21" s="4" t="n">
+      <c r="G21" s="8" t="n">
         <v>0.06614303208877151</v>
       </c>
     </row>
@@ -957,22 +1763,22 @@
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B22" s="7" t="n">
         <v>0.4771957258274694</v>
       </c>
-      <c r="C22" s="4" t="n">
+      <c r="C22" s="8" t="n">
         <v>0.4628811274289059</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" s="7" t="n">
         <v>0.438471429602897</v>
       </c>
-      <c r="E22" s="3" t="n">
+      <c r="E22" s="7" t="n">
         <v>0.1407619047619047</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" s="9" t="n">
         <v>19.78752241532008</v>
       </c>
-      <c r="G22" s="4" t="n">
+      <c r="G22" s="8" t="n">
         <v>0.06825545236370674</v>
       </c>
     </row>
@@ -980,22 +1786,22 @@
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B23" s="7" t="n">
         <v>0.4639040917383372</v>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C23" s="8" t="n">
         <v>0.4505620196464964</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" s="7" t="n">
         <v>0.4274121602213995</v>
       </c>
-      <c r="E23" s="3" t="n">
+      <c r="E23" s="7" t="n">
         <v>0.143952380952381</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" s="9" t="n">
         <v>19.80117741028468</v>
       </c>
-      <c r="G23" s="4" t="n">
+      <c r="G23" s="8" t="n">
         <v>0.07371046930850976</v>
       </c>
     </row>
@@ -1003,22 +1809,22 @@
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B24" s="7" t="n">
         <v>0.4594735470419599</v>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="C24" s="8" t="n">
         <v>0.4562442626657116</v>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" s="7" t="n">
         <v>0.4218846426309296</v>
       </c>
-      <c r="E24" s="3" t="n">
+      <c r="E24" s="7" t="n">
         <v>0.1348571428571429</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" s="9" t="n">
         <v>19.60426377058029</v>
       </c>
-      <c r="G24" s="4" t="n">
+      <c r="G24" s="8" t="n">
         <v>0.07494531696604863</v>
       </c>
     </row>
@@ -1026,22 +1832,22 @@
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B25" s="7" t="n">
         <v>0.4698983580922596</v>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="C25" s="8" t="n">
         <v>0.4608231271338195</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" s="7" t="n">
         <v>0.4288150420526599</v>
       </c>
-      <c r="E25" s="3" t="n">
+      <c r="E25" s="7" t="n">
         <v>0.1412380952380952</v>
       </c>
-      <c r="F25" s="5" t="n">
+      <c r="F25" s="9" t="n">
         <v>19.545652004083</v>
       </c>
-      <c r="G25" s="4" t="n">
+      <c r="G25" s="8" t="n">
         <v>0.07575788497726298</v>
       </c>
     </row>
@@ -1049,22 +1855,22 @@
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B26" s="7" t="n">
         <v>0.4521761793067501</v>
       </c>
-      <c r="C26" s="4" t="n">
+      <c r="C26" s="8" t="n">
         <v>0.4317262215618988</v>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" s="7" t="n">
         <v>0.4117433560152107</v>
       </c>
-      <c r="E26" s="3" t="n">
+      <c r="E26" s="7" t="n">
         <v>0.141</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" s="9" t="n">
         <v>19.61280397176743</v>
       </c>
-      <c r="G26" s="4" t="n">
+      <c r="G26" s="8" t="n">
         <v>0.07107927071281607</v>
       </c>
     </row>
@@ -1072,22 +1878,22 @@
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="3" t="n">
+      <c r="B27" s="7" t="n">
         <v>0.4670315350534271</v>
       </c>
-      <c r="C27" s="4" t="n">
+      <c r="C27" s="8" t="n">
         <v>0.4563295319761989</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" s="7" t="n">
         <v>0.4288284799659005</v>
       </c>
-      <c r="E27" s="3" t="n">
+      <c r="E27" s="7" t="n">
         <v>0.1412380952380952</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F27" s="9" t="n">
         <v>19.74820477167765</v>
       </c>
-      <c r="G27" s="4" t="n">
+      <c r="G27" s="8" t="n">
         <v>0.06857999469254483</v>
       </c>
     </row>
@@ -1095,22 +1901,22 @@
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B28" s="7" t="n">
         <v>0.4586916862131874</v>
       </c>
-      <c r="C28" s="4" t="n">
+      <c r="C28" s="8" t="n">
         <v>0.4410693978703423</v>
       </c>
-      <c r="D28" s="3" t="n">
+      <c r="D28" s="7" t="n">
         <v>0.4192767237996456</v>
       </c>
-      <c r="E28" s="3" t="n">
+      <c r="E28" s="7" t="n">
         <v>0.1393809523809524</v>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="F28" s="9" t="n">
         <v>19.68905475934347</v>
       </c>
-      <c r="G28" s="4" t="n">
+      <c r="G28" s="8" t="n">
         <v>0.07123077266751819</v>
       </c>
     </row>
@@ -1118,22 +1924,22 @@
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="3" t="n">
+      <c r="B29" s="7" t="n">
         <v>0.4659890539483972</v>
       </c>
-      <c r="C29" s="4" t="n">
+      <c r="C29" s="8" t="n">
         <v>0.4610301200749258</v>
       </c>
-      <c r="D29" s="3" t="n">
+      <c r="D29" s="7" t="n">
         <v>0.4251207433369201</v>
       </c>
-      <c r="E29" s="3" t="n">
+      <c r="E29" s="7" t="n">
         <v>0.1335238095238095</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" s="9" t="n">
         <v>19.65457094510396</v>
       </c>
-      <c r="G29" s="4" t="n">
+      <c r="G29" s="8" t="n">
         <v>0.06437136255183748</v>
       </c>
     </row>
@@ -1141,22 +1947,22 @@
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B30" s="7" t="n">
         <v>0.4560854834506124</v>
       </c>
-      <c r="C30" s="4" t="n">
+      <c r="C30" s="8" t="n">
         <v>0.445586717897399</v>
       </c>
-      <c r="D30" s="3" t="n">
+      <c r="D30" s="7" t="n">
         <v>0.4182985267620441</v>
       </c>
-      <c r="E30" s="3" t="n">
+      <c r="E30" s="7" t="n">
         <v>0.1422857142857143</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="F30" s="9" t="n">
         <v>19.7076512893041</v>
       </c>
-      <c r="G30" s="4" t="n">
+      <c r="G30" s="8" t="n">
         <v>0.07178161976541614</v>
       </c>
     </row>
@@ -1164,22 +1970,22 @@
       <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="3" t="n">
+      <c r="B31" s="7" t="n">
         <v>0.4818868908001043</v>
       </c>
-      <c r="C31" s="4" t="n">
+      <c r="C31" s="8" t="n">
         <v>0.4667553091474813</v>
       </c>
-      <c r="D31" s="3" t="n">
+      <c r="D31" s="7" t="n">
         <v>0.4431493430150057</v>
       </c>
-      <c r="E31" s="3" t="n">
+      <c r="E31" s="7" t="n">
         <v>0.1418022512627673</v>
       </c>
-      <c r="F31" s="5" t="n">
+      <c r="F31" s="9" t="n">
         <v>21.58882046143214</v>
       </c>
-      <c r="G31" s="4" t="n">
+      <c r="G31" s="8" t="n">
         <v>0.07494794105211995</v>
       </c>
     </row>
@@ -1188,7 +1994,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1237,14 +2043,14 @@
           <t>p002</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n">
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n">
         <v>0.1295282772999739</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="7" t="n">
         <v>0.9936551724137931</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="7" t="n">
         <v>0.9991724137931034</v>
       </c>
     </row>
@@ -1254,14 +2060,14 @@
           <t>p012</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n">
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n">
         <v>0.107375553818087</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="7" t="n">
         <v>0.9876063183475091</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="7" t="n">
         <v>0.9982989064398542</v>
       </c>
     </row>
@@ -1271,14 +2077,14 @@
           <t>p014</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n">
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n">
         <v>0.1032056293979672</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="7" t="n">
         <v>0.9883561643835617</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="7" t="n">
         <v>0.9997716894977169</v>
       </c>
     </row>
@@ -1288,14 +2094,14 @@
           <t>p015</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n">
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="7" t="n">
         <v>0.1183216054209017</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="7" t="n">
         <v>0.9942857142857143</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="7" t="n">
         <v>0.9997714285714285</v>
       </c>
     </row>
@@ -1305,14 +2111,14 @@
           <t>p016</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n">
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n">
         <v>0.09199895751889497</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="7" t="n">
         <v>0.9964749536178108</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" s="7" t="n">
         <v>0.9988868274582561</v>
       </c>
     </row>
@@ -1322,14 +2128,14 @@
           <t>p021</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n">
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n">
         <v>0.1751368256450352</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="7" t="n">
         <v>0.9915925626515764</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="7" t="n">
         <v>0.9978981406628941</v>
       </c>
     </row>
@@ -1339,14 +2145,14 @@
           <t>p022</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n">
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n">
         <v>0.1211884284597342</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="7" t="n">
         <v>0.9995133819951338</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="7" t="n">
         <v>0.9998377939983779</v>
       </c>
     </row>
@@ -1356,14 +2162,14 @@
           <t>p024</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n">
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n">
         <v>0.1769611675788376</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" s="7" t="n">
         <v>0.9975530179445351</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="7" t="n">
         <v>0.999510603588907</v>
       </c>
     </row>
@@ -1373,14 +2179,14 @@
           <t>p026</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n">
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n">
         <v>0.09252019807140996</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="7" t="n">
         <v>0.9953177257525083</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="7" t="n">
         <v>0.9986622073578595</v>
       </c>
     </row>
@@ -1390,14 +2196,14 @@
           <t>p035</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n">
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n">
         <v>0.1019025280166797</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="7" t="n">
         <v>0.994811320754717</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="7" t="n">
         <v>0.9955188679245283</v>
       </c>
     </row>
@@ -1407,14 +2213,14 @@
           <t>p039</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n">
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n">
         <v>0.1250977326035966</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="7" t="n">
         <v>0.9920122887864823</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="7" t="n">
         <v>0.9978494623655914</v>
       </c>
     </row>
@@ -1424,14 +2230,14 @@
           <t>p041</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n">
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n">
         <v>0.1701850403961428</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="7" t="n">
         <v>0.9963636363636363</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="7" t="n">
         <v>0.9996694214876033</v>
       </c>
     </row>
@@ -1441,14 +2247,14 @@
           <t>p042</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n">
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n">
         <v>0.1436017722178785</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="7" t="n">
         <v>0.9942470389170897</v>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E14" s="7" t="n">
         <v>0.9979695431472081</v>
       </c>
     </row>
@@ -1458,14 +2264,14 @@
           <t>p045</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n">
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n">
         <v>0.1060724524367996</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="7" t="n">
         <v>0.9953038674033149</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="7" t="n">
         <v>0.9986187845303868</v>
       </c>
     </row>
@@ -1475,14 +2281,14 @@
           <t>p047</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n">
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n">
         <v>0.1962470680218921</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="7" t="n">
         <v>0.9846706586826347</v>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E16" s="7" t="n">
         <v>0.9952095808383233</v>
       </c>
     </row>
@@ -1492,14 +2298,14 @@
           <t>p049</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n">
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n">
         <v>0.1232733906697941</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" s="7" t="n">
         <v>0.9972304648862512</v>
       </c>
-      <c r="E17" s="3" t="n">
+      <c r="E17" s="7" t="n">
         <v>0.9998021760633037</v>
       </c>
     </row>
@@ -1509,14 +2315,14 @@
           <t>p050</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n">
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n">
         <v>0.09929632525410477</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" s="7" t="n">
         <v>0.9886075949367089</v>
       </c>
-      <c r="E18" s="3" t="n">
+      <c r="E18" s="7" t="n">
         <v>0.9972151898734177</v>
       </c>
     </row>
@@ -1526,14 +2332,14 @@
           <t>p051</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n">
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n">
         <v>0.1386499869689862</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" s="7" t="n">
         <v>0.9921739130434782</v>
       </c>
-      <c r="E19" s="3" t="n">
+      <c r="E19" s="7" t="n">
         <v>0.9993478260869565</v>
       </c>
     </row>
@@ -1543,14 +2349,14 @@
           <t>p052</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n">
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="7" t="n">
         <v>0.2389887933281209</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" s="7" t="n">
         <v>0.9921621621621621</v>
       </c>
-      <c r="E20" s="3" t="n">
+      <c r="E20" s="7" t="n">
         <v>0.9978378378378379</v>
       </c>
     </row>
@@ -1560,14 +2366,14 @@
           <t>p056</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n">
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="n">
         <v>0.1743549648162627</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" s="7" t="n">
         <v>0.9899244332493703</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="E21" s="7" t="n">
         <v>0.9979848866498741</v>
       </c>
     </row>
@@ -1577,14 +2383,14 @@
           <t>p061</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n">
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="n">
         <v>0.2439405785770133</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" s="7" t="n">
         <v>0.9960444993819531</v>
       </c>
-      <c r="E22" s="3" t="n">
+      <c r="E22" s="7" t="n">
         <v>0.9977750309023485</v>
       </c>
     </row>
@@ -1593,7 +2399,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1630,7 +2436,7 @@
           <t>p064</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="7" t="n">
         <v>0.6695121951219513</v>
       </c>
       <c r="C2" s="2" t="n">
@@ -1643,7 +2449,7 @@
           <t>p066</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="7" t="n">
         <v>0.6092843326885881</v>
       </c>
       <c r="C3" s="2" t="n">
@@ -1656,7 +2462,7 @@
           <t>p072</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="7" t="n">
         <v>0.2052023121387283</v>
       </c>
       <c r="C4" s="2" t="n">
@@ -1669,7 +2475,7 @@
           <t>p075</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="7" t="n">
         <v>0.3587223587223587</v>
       </c>
       <c r="C5" s="2" t="n">
@@ -1682,7 +2488,7 @@
           <t>p081</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="7" t="n">
         <v>0.3730255164034022</v>
       </c>
       <c r="C6" s="2" t="n">
@@ -1694,7 +2500,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1725,7 +2531,7 @@
           <t>Final global student acc</t>
         </is>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="7">
         <f>Baseline_Rounds!B31</f>
         <v/>
       </c>
@@ -1736,7 +2542,7 @@
           <t>Final global student macro-F1</t>
         </is>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="8">
         <f>Baseline_Rounds!C31</f>
         <v/>
       </c>
@@ -1747,7 +2553,7 @@
           <t>Final mean private teacher acc</t>
         </is>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="7">
         <f>Baseline_Rounds!E31</f>
         <v/>
       </c>
@@ -1758,7 +2564,7 @@
           <t>Best global student acc</t>
         </is>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="7">
         <f>MAX(Baseline_Rounds!B2:B31)</f>
         <v/>
       </c>
@@ -1769,7 +2575,7 @@
           <t>Best global student macro-F1</t>
         </is>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="8">
         <f>MAX(Baseline_Rounds!C2:C31)</f>
         <v/>
       </c>
@@ -1780,7 +2586,7 @@
           <t>Best mean private teacher acc</t>
         </is>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="7">
         <f>MAX(Baseline_Rounds!E2:E31)</f>
         <v/>
       </c>
@@ -1791,7 +2597,7 @@
           <t>Final mean private teacher macro-F1</t>
         </is>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="8">
         <f>Baseline_Rounds!G31</f>
         <v/>
       </c>
@@ -1802,13 +2608,13 @@
           <t>Total training time (h)</t>
         </is>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="3">
         <f>SUM(Baseline_Rounds!F2:F31)/60</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Setting: 21 clients (one per driver; p064, p066, p072, p075, p081 held out as unseen test drivers), 30 rounds x 5 local epochs, batch 8, ViT-B mentor / ViT-S mentee, full FedKD loss, no SVD compression. Accuracy and F1 are measured on the held-out drivers.</t>
         </is>
@@ -1817,4 +2623,1032 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Run (config folder)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Final grad-match loss (best seed)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Time (min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>p002</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>p002</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>10.18981834941837</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>10.02273675431274</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>9.40250867502931</v>
+      </c>
+      <c r="H2" s="3">
+        <f>E2-G2</f>
+        <v/>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>0.1020715609192848</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>202.1691537022591</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>10.92384761775596</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>10.76693620718362</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>9.988775402453584</v>
+      </c>
+      <c r="H3" s="3">
+        <f>E3-G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>0.08336395770311356</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>206.3601462403933</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>10.65960550177276</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>10.35919985618149</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>10.14880432187795</v>
+      </c>
+      <c r="H4" s="3">
+        <f>E4-G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>0.3672726154327393</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>220.7056279460589</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>9.879232901906896</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>9.619753613356174</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>10.07038371983996</v>
+      </c>
+      <c r="H5" s="3">
+        <f>E5-G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.2159069329500198</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>186.3760811726252</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>p021</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>p021</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>10.15026036519444</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>9.839114019807274</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>9.450420919396539</v>
+      </c>
+      <c r="H6" s="3">
+        <f>E6-G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>0.5500203967094421</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>201.278364944458</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>9.769899243281543</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>9.753765040360975</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>9.082354949847025</v>
+      </c>
+      <c r="H7" s="3">
+        <f>E7-G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>0.1388921737670898</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>203.8180212457975</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Averages per setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Attacks</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only)</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>COUNTIF(A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="10">
+        <f>AVERAGEIFS(D$2:D$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="3">
+        <f>AVERAGEIFS(E$2:E$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="E11" s="3">
+        <f>AVERAGEIFS(F$2:F$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="3">
+        <f>AVERAGEIFS(G$2:G$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="3">
+        <f>AVERAGEIFS(H$2:H$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Threat model: honest-but-curious server sees one client's student gradient for one local step (batch 8, distinct labels, round-30 global student). Private teacher and projector are unknown to the attacker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>PSNR: images in [0,1], reconstructions matched one-to-one to ground truth (Hungarian), averaged over the batch. Consensus = pixel mean over seeds; best seed = lowest gradient-matching loss (attacker-selectable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Gray floor: PSNR of a uniform gray image; a reconstruction below it carries no recoverable pixel information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Run p002: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Run p012: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Run p014: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Run p015: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Run p021: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Run p035: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A123"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Each grid: row 1 = actual batch, row 2 = consensus reconstruction, row 3 = best-seed reconstruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p002 - run p002</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p012 - run p012</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p014 - run p014</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p015 - run p015</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p021 - run p021</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p035 - run p035</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Run (config folder)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Final grad-match loss (best seed)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Time (min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>p002</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>p002</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>11.95569679194365</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>11.9642847229547</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>9.40250867502931</v>
+      </c>
+      <c r="H2" s="3">
+        <f>E2-G2</f>
+        <v/>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>0.03264361619949341</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>380.7995753804843</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>12.01081569052551</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>11.82164962106386</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>9.988775402453584</v>
+      </c>
+      <c r="H3" s="3">
+        <f>E3-G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>0.03365790098905563</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>388.8103427012762</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>10.47159694146267</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>10.33662003823281</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>10.14880432187795</v>
+      </c>
+      <c r="H4" s="3">
+        <f>E4-G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>0.03335896506905556</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>417.1127759496371</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>12.00279410983525</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>11.54788435056746</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>10.07038371983996</v>
+      </c>
+      <c r="H5" s="3">
+        <f>E5-G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.02070866525173187</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>341.1732741475105</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>p021</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>p021</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>10.27059412332502</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>10.04729325639967</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>9.450420919396539</v>
+      </c>
+      <c r="H6" s="3">
+        <f>E6-G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>0.03082906268537045</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>377.3576625108719</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>9.597271589453804</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>9.647701764458878</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>9.082354949847025</v>
+      </c>
+      <c r="H7" s="3">
+        <f>E7-G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>0.01635104231536388</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>384.069699660937</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Averages per setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Attacks</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>COUNTIF(A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="10">
+        <f>AVERAGEIFS(D$2:D$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="3">
+        <f>AVERAGEIFS(E$2:E$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="E11" s="3">
+        <f>AVERAGEIFS(F$2:F$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="3">
+        <f>AVERAGEIFS(G$2:G$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="3">
+        <f>AVERAGEIFS(H$2:H$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Threat model: honest-but-curious server sees one client's student gradient for one local step (batch 8, distinct labels, round-30 global student). Private teacher and projector are unknown to the attacker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>PSNR: images in [0,1], reconstructions matched one-to-one to ground truth (Hungarian), averaged over the batch. Consensus = pixel mean over seeds; best seed = lowest gradient-matching loss (attacker-selectable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Gray floor: PSNR of a uniform gray image; a reconstruction below it carries no recoverable pixel information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Run p002: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Run p012: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Run p014: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Run p015: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Run p021: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Run p035: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A123"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Each grid: row 1 = actual batch, row 2 = consensus reconstruction, row 3 = best-seed reconstruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p002 - run p002</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p012 - run p012</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p014 - run p014</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p015 - run p015</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p021 - run p021</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p035 - run p035</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add CIFAR-100 v2 (teacher lr 1e-5, weight decay 0.05) results; Excel sheets per CIFAR baseline version with teacher overfitting gap
</commit_message>
<xml_diff>
--- a/fedkd_gia/results/fedkd_gia_results.xlsx
+++ b/fedkd_gia/results/fedkd_gia_results.xlsx
@@ -12,15 +12,18 @@
     <sheet name="Baseline_Clients" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Baseline_HeldOut" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Baseline_Summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="CIFAR100_Baseline_Rounds" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="CIFAR100_Baseline_Clients" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="CIFAR100_Baseline_Summary" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="S1_full" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="S1_full_Images" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="S2_full" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="S2_full_Images" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="S1_full_Plots" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="S2_full_Plots" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="C100_v1_Rounds" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="C100_v1_Clients" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="C100_v1_Summary" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="C100_v2_lrwd_Rounds" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="C100_v2_lrwd_Clients" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="C100_v2_lrwd_Summary" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="S1_full" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="S1_full_Images" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="S2_full" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="S2_full_Images" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="S1_full_Plots" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="S2_full_Plots" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1195,65 +1198,870 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A123"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Each grid: row 1 = actual batch, row 2 = consensus reconstruction, row 3 = best-seed reconstruction</t>
-        </is>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Global student acc on this client's local test (round 30)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Private teacher acc on its test data (not trained on)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Student acc on own training images</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Teacher acc on own training images</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Teacher overfitting gap (train - test)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>c00</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>0.7155688622754491</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>0.7711927981995499</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>0.9639909977494373</v>
+      </c>
+      <c r="F2" s="7">
+        <f>E2-C2</f>
+        <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p002 - run p002</t>
-        </is>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>c01</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>0.7425149700598802</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>0.5059880239520959</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>0.7764441110277569</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>0.9714928732183046</v>
+      </c>
+      <c r="F3" s="7">
+        <f>E3-C3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>c02</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>0.7395209580838323</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>0.5209580838323353</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>0.7689422355588897</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0.9587396849212303</v>
+      </c>
+      <c r="F4" s="7">
+        <f>E4-C4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>c03</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0.7335329341317365</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>0.4940119760479042</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0.7861965491372843</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0.9624906226556639</v>
+      </c>
+      <c r="F5" s="7">
+        <f>E5-C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>c04</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.7634730538922155</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>0.5239520958083832</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0.7696924231057765</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0.9632408102025506</v>
+      </c>
+      <c r="F6" s="7">
+        <f>E6-C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>c05</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0.7664670658682635</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>0.5359281437125748</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0.7794448612153039</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0.9617404351087772</v>
+      </c>
+      <c r="F7" s="7">
+        <f>E7-C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>c06</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0.8083832335329342</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>0.5059880239520959</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0.7884471117779445</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0.9654913728432108</v>
+      </c>
+      <c r="F8" s="7">
+        <f>E8-C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>c07</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>0.7335329341317365</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0.5059880239520959</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.7861965491372843</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0.9692423105776444</v>
+      </c>
+      <c r="F9" s="7">
+        <f>E9-C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>c08</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>0.7664670658682635</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>0.4910179640718563</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>0.7636909227306826</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>0.9624906226556639</v>
+      </c>
+      <c r="F10" s="7">
+        <f>E10-C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>c09</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0.7544910179640718</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>0.5209580838323353</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0.768192048012003</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>0.9669917479369843</v>
+      </c>
+      <c r="F11" s="7">
+        <f>E11-C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>c10</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>0.7365269461077845</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>0.5269461077844312</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>0.7524381095273819</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>0.9669917479369843</v>
+      </c>
+      <c r="F12" s="7">
+        <f>E12-C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>c11</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>0.7485029940119761</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>0.5149700598802395</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0.7666916729182296</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>0.9632408102025506</v>
+      </c>
+      <c r="F13" s="7">
+        <f>E13-C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>c12</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>0.7514970059880239</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>0.5389221556886228</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0.7809452363090773</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0.9722430607651913</v>
+      </c>
+      <c r="F14" s="7">
+        <f>E14-C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>c13</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>0.7634730538922155</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>0.5479041916167665</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0.786946736684171</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0.9624906226556639</v>
+      </c>
+      <c r="F15" s="7">
+        <f>E15-C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>c14</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>0.7574850299401198</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>0.5239520958083832</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0.7741935483870968</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0.9609902475618904</v>
+      </c>
+      <c r="F16" s="7">
+        <f>E16-C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>c15</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>0.7604790419161677</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>0.4700598802395209</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0.7801950487621906</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>0.9579894973743436</v>
+      </c>
+      <c r="F17" s="7">
+        <f>E17-C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>c16</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>0.7544910179640718</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>0.5149700598802395</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>0.7689422355588897</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>0.9684921230307577</v>
+      </c>
+      <c r="F18" s="7">
+        <f>E18-C18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>c17</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>0.7485029940119761</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>0.5179640718562875</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0.805701425356339</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>0.9632408102025506</v>
+      </c>
+      <c r="F19" s="7">
+        <f>E19-C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>c18</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>0.7874251497005988</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>0.4820359281437126</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>0.7824456114028507</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>0.9632408102025506</v>
+      </c>
+      <c r="F20" s="7">
+        <f>E20-C20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>c19</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>0.7604790419161677</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>0.4820359281437126</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>0.7756939234808702</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>0.9624906226556639</v>
+      </c>
+      <c r="F21" s="7">
+        <f>E21-C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>c20</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>0.7694610778443114</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>0.4760479041916167</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>0.7755255255255256</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>0.9572072072072072</v>
+      </c>
+      <c r="F22" s="7">
+        <f>E22-C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>c21</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>0.7095808383233533</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>0.4730538922155689</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>0.7545045045045045</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>0.9669669669669669</v>
+      </c>
+      <c r="F23" s="7">
+        <f>E23-C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>c22</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>0.7035928143712575</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>0.4670658682634731</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>0.7695195195195195</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>0.96996996996997</v>
+      </c>
+      <c r="F24" s="7">
+        <f>E24-C24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>c23</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>0.7604790419161677</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>0.5029940119760479</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>0.7725225225225225</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>0.9647147147147147</v>
+      </c>
+      <c r="F25" s="7">
+        <f>E25-C25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>c24</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>0.7544910179640718</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>0.437125748502994</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>0.7807807807807807</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>0.9632132132132132</v>
+      </c>
+      <c r="F26" s="7">
+        <f>E26-C26</f>
+        <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p012 - run p012</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p014 - run p014</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p015 - run p015</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p021 - run p021</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p035 - run p035</t>
-        </is>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>c25</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>0.7305389221556886</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>0.4790419161676647</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>0.7792792792792793</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>0.9654654654654654</v>
+      </c>
+      <c r="F27" s="7">
+        <f>E27-C27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>c26</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>0.7395209580838323</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>0.4910179640718563</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>0.7515015015015015</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>0.9714714714714715</v>
+      </c>
+      <c r="F28" s="7">
+        <f>E28-C28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>c27</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>0.7395209580838323</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>0.5059880239520959</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>0.7665165165165165</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>0.9594594594594594</v>
+      </c>
+      <c r="F29" s="7">
+        <f>E29-C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>c28</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>0.7874251497005988</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>0.4431137724550898</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>0.7815315315315315</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>0.9542042042042042</v>
+      </c>
+      <c r="F30" s="7">
+        <f>E30-C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>c29</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>0.7664670658682635</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>0.5419161676646707</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>0.7980480480480481</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>0.9677177177177178</v>
+      </c>
+      <c r="F31" s="7">
+        <f>E31-C31</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Final global student acc</t>
+        </is>
+      </c>
+      <c r="B2" s="7">
+        <f>C100_v2_lrwd_Rounds!B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Final global student macro-F1</t>
+        </is>
+      </c>
+      <c r="B3" s="8">
+        <f>C100_v2_lrwd_Rounds!C31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Final mean private teacher acc</t>
+        </is>
+      </c>
+      <c r="B4" s="7">
+        <f>C100_v2_lrwd_Rounds!E31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Best global student acc</t>
+        </is>
+      </c>
+      <c r="B5" s="7">
+        <f>MAX(C100_v2_lrwd_Rounds!B2:B31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Best global student macro-F1</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>MAX(C100_v2_lrwd_Rounds!C2:C31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Best mean private teacher acc</t>
+        </is>
+      </c>
+      <c r="B7" s="7">
+        <f>MAX(C100_v2_lrwd_Rounds!E2:E31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Final mean private teacher macro-F1</t>
+        </is>
+      </c>
+      <c r="B8" s="8">
+        <f>C100_v2_lrwd_Rounds!G31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Total training time (h)</t>
+        </is>
+      </c>
+      <c r="B9" s="3">
+        <f>SUM(C100_v2_lrwd_Rounds!F2:F31)/60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Setting: CIFAR-100, 30 IID clients (80/20 local train/test, 1,333 / 334 images each), 30 rounds x 1 local epoch, batch 8, 32x32 images upsampled to 224, ViT-B mentor / ViT-S mentee, full FedKD loss, no SVD. Global student acc/F1: official 10k test set; per-client and teacher numbers: each client's local 20% test split. v2: teacher lr 1e-5, AdamW weight decay 0.05.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1329,7 +2137,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1346,10 +2154,10 @@
         <v>0.75</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>11.95569679194365</v>
+        <v>10.18981834941837</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>11.9642847229547</v>
+        <v>10.02273675431274</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>9.40250867502931</v>
@@ -1359,16 +2167,16 @@
         <v/>
       </c>
       <c r="I2" s="8" t="n">
-        <v>0.03264361619949341</v>
+        <v>0.1020715609192848</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>380.7995753804843</v>
+        <v>202.1691537022591</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1385,10 +2193,10 @@
         <v>0.875</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>12.01081569052551</v>
+        <v>10.92384761775596</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>11.82164962106386</v>
+        <v>10.76693620718362</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>9.988775402453584</v>
@@ -1398,16 +2206,16 @@
         <v/>
       </c>
       <c r="I3" s="8" t="n">
-        <v>0.03365790098905563</v>
+        <v>0.08336395770311356</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>388.8103427012762</v>
+        <v>206.3601462403933</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1424,10 +2232,10 @@
         <v>0.75</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>10.47159694146267</v>
+        <v>10.65960550177276</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>10.33662003823281</v>
+        <v>10.35919985618149</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>10.14880432187795</v>
@@ -1437,16 +2245,16 @@
         <v/>
       </c>
       <c r="I4" s="8" t="n">
-        <v>0.03335896506905556</v>
+        <v>0.3672726154327393</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>417.1127759496371</v>
+        <v>220.7056279460589</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -1463,10 +2271,10 @@
         <v>0.75</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>12.00279410983525</v>
+        <v>9.879232901906896</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11.54788435056746</v>
+        <v>9.619753613356174</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>10.07038371983996</v>
@@ -1476,16 +2284,16 @@
         <v/>
       </c>
       <c r="I5" s="8" t="n">
-        <v>0.02070866525173187</v>
+        <v>0.2159069329500198</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>341.1732741475105</v>
+        <v>186.3760811726252</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1502,10 +2310,10 @@
         <v>0.75</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>10.27059412332502</v>
+        <v>10.15026036519444</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10.04729325639967</v>
+        <v>9.839114019807274</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>9.450420919396539</v>
@@ -1515,16 +2323,16 @@
         <v/>
       </c>
       <c r="I6" s="8" t="n">
-        <v>0.03082906268537045</v>
+        <v>0.5500203967094421</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>377.3576625108719</v>
+        <v>201.278364944458</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1541,10 +2349,10 @@
         <v>0.75</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>9.597271589453804</v>
+        <v>9.769899243281543</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>9.647701764458878</v>
+        <v>9.753765040360975</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>9.082354949847025</v>
@@ -1554,10 +2362,10 @@
         <v/>
       </c>
       <c r="I7" s="8" t="n">
-        <v>0.01635104231536388</v>
+        <v>0.1388921737670898</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>384.069699660937</v>
+        <v>203.8180212457975</v>
       </c>
     </row>
     <row r="9">
@@ -1607,7 +2415,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B11">
@@ -1703,7 +2511,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1722,42 +2530,42 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p002 - run p002</t>
+          <t>S1 no teacher (CE only) - client p002 - run p002</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p012 - run p012</t>
+          <t>S1 no teacher (CE only) - client p012 - run p012</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p014 - run p014</t>
+          <t>S1 no teacher (CE only) - client p014 - run p014</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p015 - run p015</t>
+          <t>S1 no teacher (CE only) - client p015 - run p015</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p021 - run p021</t>
+          <t>S1 no teacher (CE only) - client p021 - run p021</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p035 - run p035</t>
+          <t>S1 no teacher (CE only) - client p035 - run p035</t>
         </is>
       </c>
     </row>
@@ -1767,7 +2575,521 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Run (config folder)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Final grad-match loss (best seed)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Time (min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>p002</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>p002</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>11.95569679194365</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>11.9642847229547</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>9.40250867502931</v>
+      </c>
+      <c r="H2" s="3">
+        <f>E2-G2</f>
+        <v/>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>0.03264361619949341</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>380.7995753804843</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>12.01081569052551</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>11.82164962106386</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>9.988775402453584</v>
+      </c>
+      <c r="H3" s="3">
+        <f>E3-G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>0.03365790098905563</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>388.8103427012762</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>10.47159694146267</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>10.33662003823281</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>10.14880432187795</v>
+      </c>
+      <c r="H4" s="3">
+        <f>E4-G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>0.03335896506905556</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>417.1127759496371</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>12.00279410983525</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>11.54788435056746</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>10.07038371983996</v>
+      </c>
+      <c r="H5" s="3">
+        <f>E5-G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.02070866525173187</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>341.1732741475105</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>p021</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>p021</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>10.27059412332502</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>10.04729325639967</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>9.450420919396539</v>
+      </c>
+      <c r="H6" s="3">
+        <f>E6-G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>0.03082906268537045</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>377.3576625108719</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>9.597271589453804</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>9.647701764458878</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>9.082354949847025</v>
+      </c>
+      <c r="H7" s="3">
+        <f>E7-G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>0.01635104231536388</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>384.069699660937</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Averages per setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Attacks</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>COUNTIF(A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="10">
+        <f>AVERAGEIFS(D$2:D$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="3">
+        <f>AVERAGEIFS(E$2:E$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="E11" s="3">
+        <f>AVERAGEIFS(F$2:F$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="3">
+        <f>AVERAGEIFS(G$2:G$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="3">
+        <f>AVERAGEIFS(H$2:H$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Threat model: honest-but-curious server sees one client's student gradient for one local step (batch 8, distinct labels, round-30 global student). Private teacher and projector are unknown to the attacker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>PSNR: images in [0,1], reconstructions matched one-to-one to ground truth (Hungarian), averaged over the batch. Consensus = pixel mean over seeds; best seed = lowest gradient-matching loss (attacker-selectable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Gray floor: PSNR of a uniform gray image; a reconstruction below it carries no recoverable pixel information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Run p002: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Run p012: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Run p014: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Run p015: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Run p021: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Run p035: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A123"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Each grid: row 1 = actual batch, row 2 = consensus reconstruction, row 3 = best-seed reconstruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p002 - run p002</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p012 - run p012</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p014 - run p014</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p015 - run p015</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p021 - run p021</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p035 - run p035</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1796,7 +3118,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2581,14 +3903,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2599,22 +3922,27 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Global student test acc (round 30)</t>
+          <t>Global student acc on this client's local test (round 30)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Private teacher test acc</t>
+          <t>Private teacher acc on its test data (not trained on)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Student train acc (local)</t>
+          <t>Student acc on own training images</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Teacher train acc (local)</t>
+          <t>Teacher acc on own training images</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Teacher overfitting gap (train - test)</t>
         </is>
       </c>
     </row>
@@ -2634,6 +3962,10 @@
       <c r="E2" s="7" t="n">
         <v>0.9991724137931034</v>
       </c>
+      <c r="F2" s="7">
+        <f>E2-C2</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2651,6 +3983,10 @@
       <c r="E3" s="7" t="n">
         <v>0.9982989064398542</v>
       </c>
+      <c r="F3" s="7">
+        <f>E3-C3</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2668,6 +4004,10 @@
       <c r="E4" s="7" t="n">
         <v>0.9997716894977169</v>
       </c>
+      <c r="F4" s="7">
+        <f>E4-C4</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2685,6 +4025,10 @@
       <c r="E5" s="7" t="n">
         <v>0.9997714285714285</v>
       </c>
+      <c r="F5" s="7">
+        <f>E5-C5</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2702,6 +4046,10 @@
       <c r="E6" s="7" t="n">
         <v>0.9988868274582561</v>
       </c>
+      <c r="F6" s="7">
+        <f>E6-C6</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2719,6 +4067,10 @@
       <c r="E7" s="7" t="n">
         <v>0.9978981406628941</v>
       </c>
+      <c r="F7" s="7">
+        <f>E7-C7</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2736,6 +4088,10 @@
       <c r="E8" s="7" t="n">
         <v>0.9998377939983779</v>
       </c>
+      <c r="F8" s="7">
+        <f>E8-C8</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2753,6 +4109,10 @@
       <c r="E9" s="7" t="n">
         <v>0.999510603588907</v>
       </c>
+      <c r="F9" s="7">
+        <f>E9-C9</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2770,6 +4130,10 @@
       <c r="E10" s="7" t="n">
         <v>0.9986622073578595</v>
       </c>
+      <c r="F10" s="7">
+        <f>E10-C10</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2787,6 +4151,10 @@
       <c r="E11" s="7" t="n">
         <v>0.9955188679245283</v>
       </c>
+      <c r="F11" s="7">
+        <f>E11-C11</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2804,6 +4172,10 @@
       <c r="E12" s="7" t="n">
         <v>0.9978494623655914</v>
       </c>
+      <c r="F12" s="7">
+        <f>E12-C12</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2821,6 +4193,10 @@
       <c r="E13" s="7" t="n">
         <v>0.9996694214876033</v>
       </c>
+      <c r="F13" s="7">
+        <f>E13-C13</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2838,6 +4214,10 @@
       <c r="E14" s="7" t="n">
         <v>0.9979695431472081</v>
       </c>
+      <c r="F14" s="7">
+        <f>E14-C14</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2855,6 +4235,10 @@
       <c r="E15" s="7" t="n">
         <v>0.9986187845303868</v>
       </c>
+      <c r="F15" s="7">
+        <f>E15-C15</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2872,6 +4256,10 @@
       <c r="E16" s="7" t="n">
         <v>0.9952095808383233</v>
       </c>
+      <c r="F16" s="7">
+        <f>E16-C16</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2889,6 +4277,10 @@
       <c r="E17" s="7" t="n">
         <v>0.9998021760633037</v>
       </c>
+      <c r="F17" s="7">
+        <f>E17-C17</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2906,6 +4298,10 @@
       <c r="E18" s="7" t="n">
         <v>0.9972151898734177</v>
       </c>
+      <c r="F18" s="7">
+        <f>E18-C18</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2923,6 +4319,10 @@
       <c r="E19" s="7" t="n">
         <v>0.9993478260869565</v>
       </c>
+      <c r="F19" s="7">
+        <f>E19-C19</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2940,6 +4340,10 @@
       <c r="E20" s="7" t="n">
         <v>0.9978378378378379</v>
       </c>
+      <c r="F20" s="7">
+        <f>E20-C20</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2957,6 +4361,10 @@
       <c r="E21" s="7" t="n">
         <v>0.9979848866498741</v>
       </c>
+      <c r="F21" s="7">
+        <f>E21-C21</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2973,6 +4381,10 @@
       </c>
       <c r="E22" s="7" t="n">
         <v>0.9977750309023485</v>
+      </c>
+      <c r="F22" s="7">
+        <f>E22-C22</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3962,14 +5374,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3980,22 +5393,27 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Global student test acc (round 30)</t>
+          <t>Global student acc on this client's local test (round 30)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Private teacher test acc</t>
+          <t>Private teacher acc on its test data (not trained on)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Student train acc (local)</t>
+          <t>Student acc on own training images</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Teacher train acc (local)</t>
+          <t>Teacher acc on own training images</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Teacher overfitting gap (train - test)</t>
         </is>
       </c>
     </row>
@@ -4017,6 +5435,10 @@
       <c r="E2" s="7" t="n">
         <v>0.9587396849212303</v>
       </c>
+      <c r="F2" s="7">
+        <f>E2-C2</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4036,6 +5458,10 @@
       <c r="E3" s="7" t="n">
         <v>0.9497374343585896</v>
       </c>
+      <c r="F3" s="7">
+        <f>E3-C3</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4055,6 +5481,10 @@
       <c r="E4" s="7" t="n">
         <v>0.9579894973743436</v>
       </c>
+      <c r="F4" s="7">
+        <f>E4-C4</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4074,6 +5504,10 @@
       <c r="E5" s="7" t="n">
         <v>0.9549887471867967</v>
       </c>
+      <c r="F5" s="7">
+        <f>E5-C5</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -4093,6 +5527,10 @@
       <c r="E6" s="7" t="n">
         <v>0.95423855963991</v>
       </c>
+      <c r="F6" s="7">
+        <f>E6-C6</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4112,6 +5550,10 @@
       <c r="E7" s="7" t="n">
         <v>0.9527381845461366</v>
       </c>
+      <c r="F7" s="7">
+        <f>E7-C7</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -4131,6 +5573,10 @@
       <c r="E8" s="7" t="n">
         <v>0.9624906226556639</v>
       </c>
+      <c r="F8" s="7">
+        <f>E8-C8</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4150,6 +5596,10 @@
       <c r="E9" s="7" t="n">
         <v>0.9474868717179294</v>
       </c>
+      <c r="F9" s="7">
+        <f>E9-C9</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4169,6 +5619,10 @@
       <c r="E10" s="7" t="n">
         <v>0.9422355588897224</v>
       </c>
+      <c r="F10" s="7">
+        <f>E10-C10</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4188,6 +5642,10 @@
       <c r="E11" s="7" t="n">
         <v>0.9474868717179294</v>
       </c>
+      <c r="F11" s="7">
+        <f>E11-C11</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4207,6 +5665,10 @@
       <c r="E12" s="7" t="n">
         <v>0.9549887471867967</v>
       </c>
+      <c r="F12" s="7">
+        <f>E12-C12</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4226,6 +5688,10 @@
       <c r="E13" s="7" t="n">
         <v>0.9497374343585896</v>
       </c>
+      <c r="F13" s="7">
+        <f>E13-C13</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4245,6 +5711,10 @@
       <c r="E14" s="7" t="n">
         <v>0.9647411852963241</v>
       </c>
+      <c r="F14" s="7">
+        <f>E14-C14</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4264,6 +5734,10 @@
       <c r="E15" s="7" t="n">
         <v>0.9549887471867967</v>
       </c>
+      <c r="F15" s="7">
+        <f>E15-C15</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4283,6 +5757,10 @@
       <c r="E16" s="7" t="n">
         <v>0.9512378094523631</v>
       </c>
+      <c r="F16" s="7">
+        <f>E16-C16</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4302,6 +5780,10 @@
       <c r="E17" s="7" t="n">
         <v>0.9624906226556639</v>
       </c>
+      <c r="F17" s="7">
+        <f>E17-C17</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4321,6 +5803,10 @@
       <c r="E18" s="7" t="n">
         <v>0.945986496624156</v>
       </c>
+      <c r="F18" s="7">
+        <f>E18-C18</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4340,6 +5826,10 @@
       <c r="E19" s="7" t="n">
         <v>0.9527381845461366</v>
       </c>
+      <c r="F19" s="7">
+        <f>E19-C19</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -4359,6 +5849,10 @@
       <c r="E20" s="7" t="n">
         <v>0.9564891222805701</v>
       </c>
+      <c r="F20" s="7">
+        <f>E20-C20</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4378,6 +5872,10 @@
       <c r="E21" s="7" t="n">
         <v>0.9609902475618904</v>
       </c>
+      <c r="F21" s="7">
+        <f>E21-C21</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -4397,6 +5895,10 @@
       <c r="E22" s="7" t="n">
         <v>0.9542042042042042</v>
       </c>
+      <c r="F22" s="7">
+        <f>E22-C22</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4416,6 +5918,10 @@
       <c r="E23" s="7" t="n">
         <v>0.9632132132132132</v>
       </c>
+      <c r="F23" s="7">
+        <f>E23-C23</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -4435,6 +5941,10 @@
       <c r="E24" s="7" t="n">
         <v>0.9564564564564565</v>
       </c>
+      <c r="F24" s="7">
+        <f>E24-C24</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -4454,6 +5964,10 @@
       <c r="E25" s="7" t="n">
         <v>0.9542042042042042</v>
       </c>
+      <c r="F25" s="7">
+        <f>E25-C25</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -4473,6 +5987,10 @@
       <c r="E26" s="7" t="n">
         <v>0.9594594594594594</v>
       </c>
+      <c r="F26" s="7">
+        <f>E26-C26</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4492,6 +6010,10 @@
       <c r="E27" s="7" t="n">
         <v>0.9662162162162162</v>
       </c>
+      <c r="F27" s="7">
+        <f>E27-C27</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4511,6 +6033,10 @@
       <c r="E28" s="7" t="n">
         <v>0.9512012012012012</v>
       </c>
+      <c r="F28" s="7">
+        <f>E28-C28</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4530,6 +6056,10 @@
       <c r="E29" s="7" t="n">
         <v>0.9617117117117117</v>
       </c>
+      <c r="F29" s="7">
+        <f>E29-C29</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4549,6 +6079,10 @@
       <c r="E30" s="7" t="n">
         <v>0.9481981981981982</v>
       </c>
+      <c r="F30" s="7">
+        <f>E30-C30</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4567,6 +6101,10 @@
       </c>
       <c r="E31" s="7" t="n">
         <v>0.9587087087087087</v>
+      </c>
+      <c r="F31" s="7">
+        <f>E31-C31</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -4606,7 +6144,7 @@
         </is>
       </c>
       <c r="B2" s="7">
-        <f>CIFAR100_Baseline_Rounds!B31</f>
+        <f>C100_v1_Rounds!B31</f>
         <v/>
       </c>
     </row>
@@ -4617,7 +6155,7 @@
         </is>
       </c>
       <c r="B3" s="8">
-        <f>CIFAR100_Baseline_Rounds!C31</f>
+        <f>C100_v1_Rounds!C31</f>
         <v/>
       </c>
     </row>
@@ -4628,7 +6166,7 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>CIFAR100_Baseline_Rounds!E31</f>
+        <f>C100_v1_Rounds!E31</f>
         <v/>
       </c>
     </row>
@@ -4639,7 +6177,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>MAX(CIFAR100_Baseline_Rounds!B2:B31)</f>
+        <f>MAX(C100_v1_Rounds!B2:B31)</f>
         <v/>
       </c>
     </row>
@@ -4650,7 +6188,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>MAX(CIFAR100_Baseline_Rounds!C2:C31)</f>
+        <f>MAX(C100_v1_Rounds!C2:C31)</f>
         <v/>
       </c>
     </row>
@@ -4661,7 +6199,7 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>MAX(CIFAR100_Baseline_Rounds!E2:E31)</f>
+        <f>MAX(C100_v1_Rounds!E2:E31)</f>
         <v/>
       </c>
     </row>
@@ -4672,7 +6210,7 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <f>CIFAR100_Baseline_Rounds!G31</f>
+        <f>C100_v1_Rounds!G31</f>
         <v/>
       </c>
     </row>
@@ -4683,14 +6221,14 @@
         </is>
       </c>
       <c r="B9" s="3">
-        <f>SUM(CIFAR100_Baseline_Rounds!F2:F31)/60</f>
+        <f>SUM(C100_v1_Rounds!F2:F31)/60</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Setting: CIFAR-100, 30 IID clients (80/20 local train/test, 1,333 / 334 images each), 30 rounds x 1 local epoch, batch 8, 32x32 images upsampled to 224, ViT-B mentor / ViT-S mentee, full FedKD loss, no SVD. Global student acc/F1: official 10k test set; per-client and teacher numbers: each client's local 20% test split.</t>
+          <t>Setting: CIFAR-100, 30 IID clients (80/20 local train/test, 1,333 / 334 images each), 30 rounds x 1 local epoch, batch 8, 32x32 images upsampled to 224, ViT-B mentor / ViT-S mentee, full FedKD loss, no SVD. Global student acc/F1: official 10k test set; per-client and teacher numbers: each client's local 20% test split. v1: one learning rate 3e-5, Adam, no weight decay.</t>
         </is>
       </c>
     </row>
@@ -4705,443 +6243,743 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="37" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="33" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Setting</t>
+          <t>Round</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Global student acc</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Run (config folder)</t>
+          <t>Global student macro-F1</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Label restoration acc</t>
+          <t>Mean per-client student acc (held-out drivers for State Farm)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>PSNR consensus (dB)</t>
+          <t>Mean private teacher acc</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>PSNR best seed (dB)</t>
+          <t>Round time (min)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>PSNR gray floor (dB)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Consensus - floor (dB)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Final grad-match loss (best seed)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Time (min)</t>
+          <t>Mean private teacher macro-F1</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>p002</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>p002</t>
-        </is>
-      </c>
-      <c r="D2" s="10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>10.18981834941837</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>10.02273675431274</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>9.40250867502931</v>
-      </c>
-      <c r="H2" s="3">
-        <f>E2-G2</f>
-        <v/>
-      </c>
-      <c r="I2" s="8" t="n">
-        <v>0.1020715609192848</v>
-      </c>
-      <c r="J2" s="9" t="n">
-        <v>202.1691537022591</v>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>0.0398</v>
+      </c>
+      <c r="C2" s="8" t="n">
+        <v>0.02458082325402101</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>0.03742514970059881</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>0.04161676646706587</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>9.348750813802083</v>
+      </c>
+      <c r="G2" s="8" t="n">
+        <v>0.02397810238290942</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>p012</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>p012</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>10.92384761775596</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>10.76693620718362</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>9.988775402453584</v>
-      </c>
-      <c r="H3" s="3">
-        <f>E3-G3</f>
-        <v/>
-      </c>
-      <c r="I3" s="8" t="n">
-        <v>0.08336395770311356</v>
-      </c>
-      <c r="J3" s="9" t="n">
-        <v>206.3601462403933</v>
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>0.1246937429812353</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>0.1521956087824351</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>0.2238522954091816</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>9.273272597789765</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>0.190460006983607</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>p014</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>p014</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>10.65960550177276</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>10.35919985618149</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>10.14880432187795</v>
-      </c>
-      <c r="H4" s="3">
-        <f>E4-G4</f>
-        <v/>
-      </c>
-      <c r="I4" s="8" t="n">
-        <v>0.3672726154327393</v>
-      </c>
-      <c r="J4" s="9" t="n">
-        <v>220.7056279460589</v>
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>0.3145</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>0.285702282080827</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>0.3094810379241517</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0.3468063872255489</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>9.423418653011321</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>0.31933016351418</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>p015</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>p015</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>9.879232901906896</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>9.619753613356174</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>10.07038371983996</v>
-      </c>
-      <c r="H5" s="3">
-        <f>E5-G5</f>
-        <v/>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>0.2159069329500198</v>
-      </c>
-      <c r="J5" s="9" t="n">
-        <v>186.3760811726252</v>
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0.4155</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>0.3952074866855603</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0.4127744510978044</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0.3952095808383233</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>9.56313754717509</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>0.3717112099545594</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>p021</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>p021</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>10.15026036519444</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>9.839114019807274</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>9.450420919396539</v>
-      </c>
-      <c r="H6" s="3">
-        <f>E6-G6</f>
-        <v/>
-      </c>
-      <c r="I6" s="8" t="n">
-        <v>0.5500203967094421</v>
-      </c>
-      <c r="J6" s="9" t="n">
-        <v>201.278364944458</v>
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.4748</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>0.4571865017952586</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0.4725548902195609</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0.4087824351297404</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>9.553254469235737</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>0.3832272331547645</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>p035</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>p035</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>9.769899243281543</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>9.753765040360975</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>9.082354949847025</v>
-      </c>
-      <c r="H7" s="3">
-        <f>E7-G7</f>
-        <v/>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>0.1388921737670898</v>
-      </c>
-      <c r="J7" s="9" t="n">
-        <v>203.8180212457975</v>
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0.5304</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>0.5157809899905554</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0.5270459081836326</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0.4199600798403192</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>9.566774805386862</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>0.3954177084399059</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>0.5455043767493802</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0.558183632734531</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0.4442115768463075</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>9.748437408606211</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>0.4185571937907326</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Averages per setting</t>
-        </is>
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>0.5857</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>0.5747526063398218</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.5873253493013971</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0.4459081836327346</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>9.674061985810598</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>0.4217959564263954</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>Attacks</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>Label restoration acc</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>PSNR consensus (dB)</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>PSNR best seed (dB)</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>PSNR gray floor (dB)</t>
-        </is>
-      </c>
-      <c r="G10" s="1" t="inlineStr">
-        <is>
-          <t>Consensus - floor (dB)</t>
-        </is>
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>0.6076</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>0.5988600721068893</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>0.604191616766467</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>0.4693612774451098</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>9.803691256046296</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>0.4452597475303341</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B11">
-        <f>COUNTIF(A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="C11" s="10">
-        <f>AVERAGEIFS(D$2:D$7,A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="D11" s="3">
-        <f>AVERAGEIFS(E$2:E$7,A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="E11" s="3">
-        <f>AVERAGEIFS(F$2:F$7,A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="F11" s="3">
-        <f>AVERAGEIFS(G$2:G$7,A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="G11" s="3">
-        <f>AVERAGEIFS(H$2:H$7,A$2:A$7,A11)</f>
-        <v/>
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0.628</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>0.6216599663461509</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0.6245508982035927</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>0.4695608782435131</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>9.745298043886821</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>0.4430067432094621</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>0.6443</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>0.6380230755157225</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>0.6408183632734531</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>0.4837325349301398</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>9.710044868787129</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>0.4586731188201195</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Threat model: honest-but-curious server sees one client's student gradient for one local step (batch 8, distinct labels, round-30 global student). Private teacher and projector are unknown to the attacker.</t>
-        </is>
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>0.6521</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>0.6452065528762351</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0.651696606786427</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>0.4826347305389222</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>9.720775183041891</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>0.4562807311031375</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>PSNR: images in [0,1], reconstructions matched one-to-one to ground truth (Hungarian), averaged over the batch. Consensus = pixel mean over seeds; best seed = lowest gradient-matching loss (attacker-selectable).</t>
-        </is>
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>0.6663</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>0.6627538196635772</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0.6622754491017965</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0.4860279441117764</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>9.716302768389385</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>0.461194149127668</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Gray floor: PSNR of a uniform gray image; a reconstruction below it carries no recoverable pixel information.</t>
-        </is>
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>0.678</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>0.6734525334998467</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0.67375249500998</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0.4954091816367265</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>9.801102137565612</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>0.4691565127553768</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Run p002: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>0.6834</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>0.6796334582965798</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0.6817365269461079</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0.4900199600798404</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>9.786925105253856</v>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>0.4653044217047616</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Run p012: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>0.6911</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>0.6877926011555668</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0.6905189620758486</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>0.5001996007984032</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>9.737451271216075</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>0.4778252734383999</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Run p014: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>0.6983</v>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>0.6950744247217383</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>0.6967065868263476</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>0.5027944111776448</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>9.912858684857687</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>0.4808025926981131</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Run p015: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>0.7044</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>0.7023444764174991</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0.7033932135728542</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>0.5030938123752494</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>9.961191372076671</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>0.482221824422335</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Run p021: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>0.7134</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>0.7115070227001619</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>0.710179640718563</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>0.5006986027944113</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>10.04072852134705</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>0.475918102770129</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Run p035: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>0.7154</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>0.7135000641265085</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>0.7141716566866267</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>0.5036926147704591</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>10.09966814120611</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>0.4821288618881923</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>0.724</v>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>0.7216737410189531</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>0.7187624750499002</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>0.500998003992016</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>10.03956276973089</v>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>0.4786904868469815</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>0.7266</v>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>0.725075880770674</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>0.7278443113772455</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>0.5012974051896207</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>10.05284260511398</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>0.4815010320959857</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>0.7307</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>0.7292535272203808</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>0.7302395209580838</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>0.5148702594810379</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>10.16156870126724</v>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>0.4955438508516325</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>0.7326</v>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>0.7308910000106907</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>0.7349301397205589</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>0.4981037924151696</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>10.21717770894369</v>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>0.4777646984090327</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>0.7401</v>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>0.7385189755488439</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>0.7359281437125749</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>0.5073852295409182</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>10.22765514850616</v>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>0.4894902369022373</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>0.7408</v>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>0.7401221865377292</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>0.7397205588822354</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>0.5162674650698603</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>10.26444752216339</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>0.4970155523624413</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>0.7438</v>
+      </c>
+      <c r="C28" s="8" t="n">
+        <v>0.7422062447086174</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>0.7440119760479043</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>0.5140718562874251</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>10.29801479578018</v>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>0.4939236132802999</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>0.747</v>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>0.7460747793565784</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>0.7458083832335328</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>0.5121756487025948</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>10.2890757282575</v>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>0.4937357469087499</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>0.7499</v>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>0.7490024384281952</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>0.7491017964071854</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>0.5089820359281437</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>10.30421717961629</v>
+      </c>
+      <c r="G30" s="8" t="n">
+        <v>0.4875857320897662</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>0.7497</v>
+      </c>
+      <c r="C31" s="8" t="n">
+        <v>0.7484697860906806</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>0.7517964071856287</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>0.5013972055888224</v>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>10.32751207749049</v>
+      </c>
+      <c r="G31" s="8" t="n">
+        <v>0.4810868602073491</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add CIFAR-100 v3 baseline (teacher: last 2 blocks trained, lr 1e-5, weight decay 0.05)
</commit_message>
<xml_diff>
--- a/fedkd_gia/results/fedkd_gia_results.xlsx
+++ b/fedkd_gia/results/fedkd_gia_results.xlsx
@@ -18,12 +18,15 @@
     <sheet name="C100_v2_lrwd_Rounds" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="C100_v2_lrwd_Clients" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="C100_v2_lrwd_Summary" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="S1_full" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="S1_full_Images" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="S2_full" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="S2_full_Images" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="S1_full_Plots" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="S2_full_Plots" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="C100_v3_frozen_Rounds" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="C100_v3_frozen_Clients" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="C100_v3_frozen_Summary" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="S1_full" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="S1_full_Images" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="S2_full" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="S2_full_Images" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="S1_full_Plots" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="S2_full_Plots" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2067,443 +2070,743 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="37" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="33" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Setting</t>
+          <t>Round</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Global student acc</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Run (config folder)</t>
+          <t>Global student macro-F1</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Label restoration acc</t>
+          <t>Mean per-client student acc (held-out drivers for State Farm)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>PSNR consensus (dB)</t>
+          <t>Mean private teacher acc</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>PSNR best seed (dB)</t>
+          <t>Round time (min)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>PSNR gray floor (dB)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Consensus - floor (dB)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Final grad-match loss (best seed)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Time (min)</t>
+          <t>Mean private teacher macro-F1</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>p002</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>p002</t>
-        </is>
-      </c>
-      <c r="D2" s="10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>10.18981834941837</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>10.02273675431274</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>9.40250867502931</v>
-      </c>
-      <c r="H2" s="3">
-        <f>E2-G2</f>
-        <v/>
-      </c>
-      <c r="I2" s="8" t="n">
-        <v>0.1020715609192848</v>
-      </c>
-      <c r="J2" s="9" t="n">
-        <v>202.1691537022591</v>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>0.0468</v>
+      </c>
+      <c r="C2" s="8" t="n">
+        <v>0.03189185840167265</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>0.05149700598802395</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>0.09770459081836327</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>6.111850873629252</v>
+      </c>
+      <c r="G2" s="8" t="n">
+        <v>0.08274583445064332</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>p012</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>p012</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>10.92384761775596</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>10.76693620718362</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>9.988775402453584</v>
-      </c>
-      <c r="H3" s="3">
-        <f>E3-G3</f>
-        <v/>
-      </c>
-      <c r="I3" s="8" t="n">
-        <v>0.08336395770311356</v>
-      </c>
-      <c r="J3" s="9" t="n">
-        <v>206.3601462403933</v>
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>0.1684</v>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>0.1325516864987036</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>0.1644710578842315</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>0.4240518962075849</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>6.364497701327006</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>0.3993607464831923</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>p014</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>p014</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>10.65960550177276</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>10.35919985618149</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>10.14880432187795</v>
-      </c>
-      <c r="H4" s="3">
-        <f>E4-G4</f>
-        <v/>
-      </c>
-      <c r="I4" s="8" t="n">
-        <v>0.3672726154327393</v>
-      </c>
-      <c r="J4" s="9" t="n">
-        <v>220.7056279460589</v>
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>0.3167</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>0.2878690913218188</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>0.3146706586826348</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0.6052894211576846</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>6.37537069718043</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>0.590688739038739</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>p015</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>p015</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>9.879232901906896</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>9.619753613356174</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>10.07038371983996</v>
-      </c>
-      <c r="H5" s="3">
-        <f>E5-G5</f>
-        <v/>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>0.2159069329500198</v>
-      </c>
-      <c r="J5" s="9" t="n">
-        <v>186.3760811726252</v>
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0.4119</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>0.3868002057179964</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0.4102794411177645</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0.6630738522954093</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>6.52446893453598</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>0.6515473637473638</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>p021</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>p021</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>10.15026036519444</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>9.839114019807274</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>9.450420919396539</v>
-      </c>
-      <c r="H6" s="3">
-        <f>E6-G6</f>
-        <v/>
-      </c>
-      <c r="I6" s="8" t="n">
-        <v>0.5500203967094421</v>
-      </c>
-      <c r="J6" s="9" t="n">
-        <v>201.278364944458</v>
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.4685</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>0.4462389641600082</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0.4670658682634731</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0.6711576846307385</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>6.592817596594492</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>0.6578025234025234</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>p035</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>p035</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>9.769899243281543</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>9.753765040360975</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>9.082354949847025</v>
-      </c>
-      <c r="H7" s="3">
-        <f>E7-G7</f>
-        <v/>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>0.1388921737670898</v>
-      </c>
-      <c r="J7" s="9" t="n">
-        <v>203.8180212457975</v>
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0.5211</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>0.502344064620601</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0.5144710578842315</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0.6729540918163672</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>6.553343506654103</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>0.6585116402116403</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0.5558</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>0.5433634146844951</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0.5483033932135727</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0.6759481037924151</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>6.679539887110392</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>0.6607410395160395</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Averages per setting</t>
-        </is>
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>0.5826</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>0.5725878688942736</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.5769461077844311</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0.6820359281437126</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>6.788252691427867</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>0.6665321326821325</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>Attacks</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>Label restoration acc</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>PSNR consensus (dB)</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>PSNR best seed (dB)</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>PSNR gray floor (dB)</t>
-        </is>
-      </c>
-      <c r="G10" s="1" t="inlineStr">
-        <is>
-          <t>Consensus - floor (dB)</t>
-        </is>
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>0.5968</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>0.5875056344678893</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>0.5977045908183632</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>0.6853293413173652</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>6.898306596279144</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>0.6698707218707217</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B11">
-        <f>COUNTIF(A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="C11" s="10">
-        <f>AVERAGEIFS(D$2:D$7,A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="D11" s="3">
-        <f>AVERAGEIFS(E$2:E$7,A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="E11" s="3">
-        <f>AVERAGEIFS(F$2:F$7,A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="F11" s="3">
-        <f>AVERAGEIFS(G$2:G$7,A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="G11" s="3">
-        <f>AVERAGEIFS(H$2:H$7,A$2:A$7,A11)</f>
-        <v/>
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0.6168</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>0.6102280308550402</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0.6170658682634731</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>0.6916167664670659</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>6.822972810268402</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>0.6759206608206606</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>0.6353</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>0.6282863094630726</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>0.6328343313373253</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>0.6959081836327348</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>6.962361184755961</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>0.6798005346505346</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Threat model: honest-but-curious server sees one client's student gradient for one local step (batch 8, distinct labels, round-30 global student). Private teacher and projector are unknown to the attacker.</t>
-        </is>
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>0.6437</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>0.637087143025348</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0.646506986027944</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>0.7027944111776449</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>7.01077577273051</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>0.6887213749213749</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>PSNR: images in [0,1], reconstructions matched one-to-one to ground truth (Hungarian), averaged over the batch. Consensus = pixel mean over seeds; best seed = lowest gradient-matching loss (attacker-selectable).</t>
-        </is>
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>0.6563</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>0.652109455830531</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0.6612774451097804</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0.7082834331337327</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>6.950837588310241</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>0.6937324823324822</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Gray floor: PSNR of a uniform gray image; a reconstruction below it carries no recoverable pixel information.</t>
-        </is>
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>0.6626827760085385</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0.6725548902195607</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0.7107784431137725</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>6.917064046859741</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>0.6959330983830986</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Run p002: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>0.6748</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>0.6708279773390473</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0.6785429141716569</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0.7125748502994012</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>6.955342650413513</v>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>0.6983076664076664</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Run p012: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>0.6854</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>0.6820095812484189</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0.6849301397205588</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>0.7186626746506986</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>7.037719508012136</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>0.7057672659584425</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Run p014: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>0.6918</v>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>0.6881558769442574</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>0.6953093812375252</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>0.7166666666666667</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>7.068615098794301</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>0.7029292540792541</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Run p015: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>0.6986</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>0.6965394663859175</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0.6999001996007983</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>0.7164670658682635</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>7.105815136432648</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>0.7032037516949282</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Run p021: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>0.7026</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>0.7007528262716027</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>0.7058882235528942</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>0.7248502994011978</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>7.192413874467214</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>0.7111178321678321</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Run p035: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>0.706</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>0.7038478840254503</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>0.7105788423153693</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>0.720858283433134</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>7.161082776387532</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>0.707136099086099</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>0.7113</v>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>0.7090456243365805</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>0.7155688622754492</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>0.7269461077844314</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>7.262655329704285</v>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>0.7131632497132496</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>0.7185</v>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>0.7165410566715255</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>0.7217564870259481</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>0.7301397205588824</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>7.287683208783467</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>0.7168040478040479</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>0.7232</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>0.7222449263216132</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>0.7278443113772455</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>0.7318363273453092</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>7.237768669923146</v>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>0.7189956284456284</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>0.7268</v>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>0.7254883246983453</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>0.7291417165668664</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>0.7334331337325352</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>7.239888175328573</v>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>0.721623158323158</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>0.7322</v>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>0.7309306811400842</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>0.7337325349301397</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>0.7376247504990019</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>7.309816861152649</v>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>0.7252785520035521</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>0.7357</v>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>0.7347189587958916</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>0.7359281437125749</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>0.734930139720559</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>7.351772530873617</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>0.7230128871128871</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>0.7363</v>
+      </c>
+      <c r="C28" s="8" t="n">
+        <v>0.7344844243043122</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>0.7387225548902197</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>0.7397205588822353</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>7.238454115390778</v>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>0.7267440836940834</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>0.7413999999999999</v>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>0.7403832968060364</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>0.7422155688622756</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>0.7420159680638724</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>7.241907544930776</v>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>0.7298155733155732</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>0.7442</v>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>0.743717297257055</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>0.7442115768463075</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>0.7405189620758483</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>7.267353216807048</v>
+      </c>
+      <c r="G30" s="8" t="n">
+        <v>0.7284212232212234</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>0.7468</v>
+      </c>
+      <c r="C31" s="8" t="n">
+        <v>0.7459803787570736</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>0.7476047904191618</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>0.7426147704590819</v>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>7.346505316098531</v>
+      </c>
+      <c r="G31" s="8" t="n">
+        <v>0.7301751711251713</v>
       </c>
     </row>
   </sheetData>
@@ -2517,65 +2820,870 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A123"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Each grid: row 1 = actual batch, row 2 = consensus reconstruction, row 3 = best-seed reconstruction</t>
-        </is>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Global student acc on this client's local test (round 30)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Private teacher acc on its test data (not trained on)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Student acc on own training images</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Teacher acc on own training images</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Teacher overfitting gap (train - test)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>c00</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>0.7005988023952096</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>0.7095808383233533</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>0.7809452363090773</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>0.9909977494373593</v>
+      </c>
+      <c r="F2" s="7">
+        <f>E2-C2</f>
+        <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p002 - run p002</t>
-        </is>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>c01</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>0.7335329341317365</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>0.7724550898203593</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>0.7809452363090773</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>0.9879969992498124</v>
+      </c>
+      <c r="F3" s="7">
+        <f>E3-C3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>c02</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>0.7574850299401198</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>0.7305389221556886</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>0.7764441110277569</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>0.9954988747186797</v>
+      </c>
+      <c r="F4" s="7">
+        <f>E4-C4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>c03</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0.7485029940119761</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>0.7724550898203593</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0.7696924231057765</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0.991747936984246</v>
+      </c>
+      <c r="F5" s="7">
+        <f>E5-C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>c04</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.7724550898203593</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>0.8023952095808383</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>0.7591897974493623</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0.9924981245311327</v>
+      </c>
+      <c r="F6" s="7">
+        <f>E6-C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>c05</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0.7455089820359282</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>0.7305389221556886</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0.7846961740435109</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0.9932483120780196</v>
+      </c>
+      <c r="F7" s="7">
+        <f>E7-C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>c06</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0.7694610778443114</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>0.7425149700598802</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0.7794448612153039</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0.9954988747186797</v>
+      </c>
+      <c r="F8" s="7">
+        <f>E8-C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>c07</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>0.7425149700598802</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0.7784431137724551</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.7839459864966242</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0.9924981245311327</v>
+      </c>
+      <c r="F9" s="7">
+        <f>E9-C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>c08</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>0.7514970059880239</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>0.7365269461077845</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>0.7884471117779445</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>0.9932483120780196</v>
+      </c>
+      <c r="F10" s="7">
+        <f>E10-C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>c09</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0.7455089820359282</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>0.7305389221556886</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0.7726931732933233</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>0.9924981245311327</v>
+      </c>
+      <c r="F11" s="7">
+        <f>E11-C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>c10</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>0.7335329341317365</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>0.7485029940119761</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>0.759939984996249</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>0.9902475618904726</v>
+      </c>
+      <c r="F12" s="7">
+        <f>E12-C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>c11</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>0.7455089820359282</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>0.718562874251497</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0.7629407351837959</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>0.9909977494373593</v>
+      </c>
+      <c r="F13" s="7">
+        <f>E13-C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>c12</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>0.7514970059880239</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>0.7514970059880239</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0.7771942985746436</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0.9924981245311327</v>
+      </c>
+      <c r="F14" s="7">
+        <f>E14-C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>c13</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>0.7844311377245509</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>0.7305389221556886</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0.8042010502625656</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0.9909977494373593</v>
+      </c>
+      <c r="F15" s="7">
+        <f>E15-C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>c14</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>0.7395209580838323</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>0.7155688622754491</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0.7839459864966242</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0.9879969992498124</v>
+      </c>
+      <c r="F16" s="7">
+        <f>E16-C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>c15</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>0.7514970059880239</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>0.7544910179640718</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0.7764441110277569</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>0.9939984996249063</v>
+      </c>
+      <c r="F17" s="7">
+        <f>E17-C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>c16</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>0.7574850299401198</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>0.7455089820359282</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>0.7749437359339835</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>0.9939984996249063</v>
+      </c>
+      <c r="F18" s="7">
+        <f>E18-C18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>c17</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>0.7694610778443114</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>0.7485029940119761</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0.7794448612153039</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>0.9954988747186797</v>
+      </c>
+      <c r="F19" s="7">
+        <f>E19-C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>c18</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>0.7574850299401198</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>0.7365269461077845</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>0.7996999249812453</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>0.986496624156039</v>
+      </c>
+      <c r="F20" s="7">
+        <f>E20-C20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>c19</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>0.7514970059880239</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>0.7305389221556886</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>0.7801950487621906</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>0.9909977494373593</v>
+      </c>
+      <c r="F21" s="7">
+        <f>E21-C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>c20</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>0.7604790419161677</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>0.7874251497005988</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>0.7672672672672672</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>0.9902402402402403</v>
+      </c>
+      <c r="F22" s="7">
+        <f>E22-C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>c21</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>0.7215568862275449</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>0.7035928143712575</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>0.7687687687687688</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>0.993993993993994</v>
+      </c>
+      <c r="F23" s="7">
+        <f>E23-C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>c22</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>0.7245508982035929</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>0.6946107784431138</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>0.7717717717717718</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>0.9924924924924925</v>
+      </c>
+      <c r="F24" s="7">
+        <f>E24-C24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>c23</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>0.7395209580838323</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>0.7874251497005988</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>0.7897897897897898</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>0.9902402402402403</v>
+      </c>
+      <c r="F25" s="7">
+        <f>E25-C25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>c24</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>0.7305389221556886</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>0.6976047904191617</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>0.7927927927927928</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>0.9947447447447447</v>
+      </c>
+      <c r="F26" s="7">
+        <f>E26-C26</f>
+        <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p012 - run p012</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p014 - run p014</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p015 - run p015</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p021 - run p021</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p035 - run p035</t>
-        </is>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>c25</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>0.7275449101796407</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>0.7035928143712575</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>0.9917417417417418</v>
+      </c>
+      <c r="F27" s="7">
+        <f>E27-C27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>c26</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>0.7275449101796407</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>0.7724550898203593</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>0.7417417417417418</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>0.9924924924924925</v>
+      </c>
+      <c r="F28" s="7">
+        <f>E28-C28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>c27</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>0.7245508982035929</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>0.7305389221556886</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>0.7755255255255256</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>0.9932432432432432</v>
+      </c>
+      <c r="F29" s="7">
+        <f>E29-C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>c28</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>0.7694610778443114</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>0.7604790419161677</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>0.990990990990991</v>
+      </c>
+      <c r="F30" s="7">
+        <f>E30-C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>c29</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>0.7934131736526946</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>0.7544910179640718</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>0.7905405405405406</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>0.9932432432432432</v>
+      </c>
+      <c r="F31" s="7">
+        <f>E31-C31</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Final global student acc</t>
+        </is>
+      </c>
+      <c r="B2" s="7">
+        <f>C100_v3_frozen_Rounds!B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Final global student macro-F1</t>
+        </is>
+      </c>
+      <c r="B3" s="8">
+        <f>C100_v3_frozen_Rounds!C31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Final mean private teacher acc</t>
+        </is>
+      </c>
+      <c r="B4" s="7">
+        <f>C100_v3_frozen_Rounds!E31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Best global student acc</t>
+        </is>
+      </c>
+      <c r="B5" s="7">
+        <f>MAX(C100_v3_frozen_Rounds!B2:B31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Best global student macro-F1</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>MAX(C100_v3_frozen_Rounds!C2:C31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Best mean private teacher acc</t>
+        </is>
+      </c>
+      <c r="B7" s="7">
+        <f>MAX(C100_v3_frozen_Rounds!E2:E31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Final mean private teacher macro-F1</t>
+        </is>
+      </c>
+      <c r="B8" s="8">
+        <f>C100_v3_frozen_Rounds!G31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Total training time (h)</t>
+        </is>
+      </c>
+      <c r="B9" s="3">
+        <f>SUM(C100_v3_frozen_Rounds!F2:F31)/60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Setting: CIFAR-100, 30 IID clients (80/20 local train/test, 1,333 / 334 images each), 30 rounds x 1 local epoch, batch 8, 32x32 images upsampled to 224, ViT-B mentor / ViT-S mentee, full FedKD loss, no SVD. Global student acc/F1: official 10k test set; per-client and teacher numbers: each client's local 20% test split. v3: as v2, plus only the last 2 teacher blocks (+ norm, head) trained.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2651,7 +3759,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -2668,10 +3776,10 @@
         <v>0.75</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>11.95569679194365</v>
+        <v>10.18981834941837</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>11.9642847229547</v>
+        <v>10.02273675431274</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>9.40250867502931</v>
@@ -2681,16 +3789,16 @@
         <v/>
       </c>
       <c r="I2" s="8" t="n">
-        <v>0.03264361619949341</v>
+        <v>0.1020715609192848</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>380.7995753804843</v>
+        <v>202.1691537022591</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -2707,10 +3815,10 @@
         <v>0.875</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>12.01081569052551</v>
+        <v>10.92384761775596</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>11.82164962106386</v>
+        <v>10.76693620718362</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>9.988775402453584</v>
@@ -2720,16 +3828,16 @@
         <v/>
       </c>
       <c r="I3" s="8" t="n">
-        <v>0.03365790098905563</v>
+        <v>0.08336395770311356</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>388.8103427012762</v>
+        <v>206.3601462403933</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -2746,10 +3854,10 @@
         <v>0.75</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>10.47159694146267</v>
+        <v>10.65960550177276</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>10.33662003823281</v>
+        <v>10.35919985618149</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>10.14880432187795</v>
@@ -2759,16 +3867,16 @@
         <v/>
       </c>
       <c r="I4" s="8" t="n">
-        <v>0.03335896506905556</v>
+        <v>0.3672726154327393</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>417.1127759496371</v>
+        <v>220.7056279460589</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -2785,10 +3893,10 @@
         <v>0.75</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>12.00279410983525</v>
+        <v>9.879232901906896</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11.54788435056746</v>
+        <v>9.619753613356174</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>10.07038371983996</v>
@@ -2798,16 +3906,16 @@
         <v/>
       </c>
       <c r="I5" s="8" t="n">
-        <v>0.02070866525173187</v>
+        <v>0.2159069329500198</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>341.1732741475105</v>
+        <v>186.3760811726252</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -2824,10 +3932,10 @@
         <v>0.75</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>10.27059412332502</v>
+        <v>10.15026036519444</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10.04729325639967</v>
+        <v>9.839114019807274</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>9.450420919396539</v>
@@ -2837,16 +3945,16 @@
         <v/>
       </c>
       <c r="I6" s="8" t="n">
-        <v>0.03082906268537045</v>
+        <v>0.5500203967094421</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>377.3576625108719</v>
+        <v>201.278364944458</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -2863,10 +3971,10 @@
         <v>0.75</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>9.597271589453804</v>
+        <v>9.769899243281543</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>9.647701764458878</v>
+        <v>9.753765040360975</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>9.082354949847025</v>
@@ -2876,10 +3984,10 @@
         <v/>
       </c>
       <c r="I7" s="8" t="n">
-        <v>0.01635104231536388</v>
+        <v>0.1388921737670898</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>384.069699660937</v>
+        <v>203.8180212457975</v>
       </c>
     </row>
     <row r="9">
@@ -2929,7 +4037,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B11">
@@ -3025,7 +4133,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3044,71 +4152,42 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p002 - run p002</t>
+          <t>S1 no teacher (CE only) - client p002 - run p002</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p012 - run p012</t>
+          <t>S1 no teacher (CE only) - client p012 - run p012</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p014 - run p014</t>
+          <t>S1 no teacher (CE only) - client p014 - run p014</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p015 - run p015</t>
+          <t>S1 no teacher (CE only) - client p015 - run p015</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p021 - run p021</t>
+          <t>S1 no teacher (CE only) - client p021 - run p021</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p035 - run p035</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>psnr_gain_all_clients.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>psnr_gain_vs_iteration.png</t>
+          <t>S1 no teacher (CE only) - client p035 - run p035</t>
         </is>
       </c>
     </row>
@@ -3119,6 +4198,520 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Run (config folder)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Final grad-match loss (best seed)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Time (min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>p002</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>p002</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>11.95569679194365</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>11.9642847229547</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>9.40250867502931</v>
+      </c>
+      <c r="H2" s="3">
+        <f>E2-G2</f>
+        <v/>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>0.03264361619949341</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>380.7995753804843</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>12.01081569052551</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>11.82164962106386</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>9.988775402453584</v>
+      </c>
+      <c r="H3" s="3">
+        <f>E3-G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>0.03365790098905563</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>388.8103427012762</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>10.47159694146267</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>10.33662003823281</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>10.14880432187795</v>
+      </c>
+      <c r="H4" s="3">
+        <f>E4-G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>0.03335896506905556</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>417.1127759496371</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>12.00279410983525</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>11.54788435056746</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>10.07038371983996</v>
+      </c>
+      <c r="H5" s="3">
+        <f>E5-G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.02070866525173187</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>341.1732741475105</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>p021</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>p021</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>10.27059412332502</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>10.04729325639967</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>9.450420919396539</v>
+      </c>
+      <c r="H6" s="3">
+        <f>E6-G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>0.03082906268537045</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>377.3576625108719</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>9.597271589453804</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>9.647701764458878</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>9.082354949847025</v>
+      </c>
+      <c r="H7" s="3">
+        <f>E7-G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>0.01635104231536388</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>384.069699660937</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Averages per setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Attacks</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>COUNTIF(A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="10">
+        <f>AVERAGEIFS(D$2:D$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="3">
+        <f>AVERAGEIFS(E$2:E$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="E11" s="3">
+        <f>AVERAGEIFS(F$2:F$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="3">
+        <f>AVERAGEIFS(G$2:G$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="3">
+        <f>AVERAGEIFS(H$2:H$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Threat model: honest-but-curious server sees one client's student gradient for one local step (batch 8, distinct labels, round-30 global student). Private teacher and projector are unknown to the attacker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>PSNR: images in [0,1], reconstructions matched one-to-one to ground truth (Hungarian), averaged over the batch. Consensus = pixel mean over seeds; best seed = lowest gradient-matching loss (attacker-selectable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Gray floor: PSNR of a uniform gray image; a reconstruction below it carries no recoverable pixel information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Run p002: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Run p012: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Run p014: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Run p015: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Run p021: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Run p035: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A123"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Each grid: row 1 = actual batch, row 2 = consensus reconstruction, row 3 = best-seed reconstruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p002 - run p002</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p012 - run p012</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p014 - run p014</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p015 - run p015</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p021 - run p021</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p035 - run p035</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3897,6 +5490,35 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_all_clients.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_vs_iteration.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add CIFAR-100 v3 GradInversion results (S1, S2, 20k iterations, clients c00-c03)
</commit_message>
<xml_diff>
--- a/fedkd_gia/results/fedkd_gia_results.xlsx
+++ b/fedkd_gia/results/fedkd_gia_results.xlsx
@@ -21,12 +21,18 @@
     <sheet name="C100_v3_frozen_Rounds" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="C100_v3_frozen_Clients" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="C100_v3_frozen_Summary" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="S1_full" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="S1_full_Images" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="S2_full" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="S2_full_Images" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="S1_full_Plots" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="S2_full_Plots" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="CIFAR_v3_S1_full" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="CIFAR_v3_S1_full_Images" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="CIFAR_v3_S2_full" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="CIFAR_v3_S2_full_Images" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="S1_full" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="S1_full_Images" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="S2_full" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="S2_full_Images" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="CIFAR_v3_S1_full_Plots" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="CIFAR_v3_S2_full_Plots" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="S1_full_Plots" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="S2_full_Plots" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -277,21 +283,26 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>99</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10477500" cy="3924300"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
+        <a:blip cstate="print" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -306,17 +317,67 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>123</row>
+      <row>27</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="10477500" cy="3924300"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>75</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -330,7 +391,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -485,7 +546,162 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>75</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>99</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>123</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -540,7 +756,117 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4819650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4276725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4819650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4276725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -3689,7 +4015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3764,35 +4090,35 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>p002</t>
+          <t>c00</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>p002</t>
+          <t>c00</t>
         </is>
       </c>
       <c r="D2" s="10" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>10.18981834941837</v>
+        <v>13.98089330915437</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>10.02273675431274</v>
+        <v>13.5410380407718</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>9.40250867502931</v>
+        <v>12.34300487756501</v>
       </c>
       <c r="H2" s="3">
         <f>E2-G2</f>
         <v/>
       </c>
       <c r="I2" s="8" t="n">
-        <v>0.1020715609192848</v>
+        <v>0.1715378612279892</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>202.1691537022591</v>
+        <v>208.2643643458684</v>
       </c>
     </row>
     <row r="3">
@@ -3803,35 +4129,35 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>p012</t>
+          <t>c01</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>p012</t>
+          <t>c01</t>
         </is>
       </c>
       <c r="D3" s="10" t="n">
-        <v>0.875</v>
+        <v>0.625</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>10.92384761775596</v>
+        <v>12.31230298512068</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>10.76693620718362</v>
+        <v>12.43724754995335</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>9.988775402453584</v>
+        <v>10.39194379566542</v>
       </c>
       <c r="H3" s="3">
         <f>E3-G3</f>
         <v/>
       </c>
       <c r="I3" s="8" t="n">
-        <v>0.08336395770311356</v>
+        <v>0.2176778316497803</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>206.3601462403933</v>
+        <v>209.9841281096141</v>
       </c>
     </row>
     <row r="4">
@@ -3842,35 +4168,35 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>p014</t>
+          <t>c02</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>p014</t>
+          <t>c02</t>
         </is>
       </c>
       <c r="D4" s="10" t="n">
-        <v>0.75</v>
+        <v>0.625</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>10.65960550177276</v>
+        <v>14.98678517499856</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>10.35919985618149</v>
+        <v>14.87393583342539</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>10.14880432187795</v>
+        <v>12.68074810257826</v>
       </c>
       <c r="H4" s="3">
         <f>E4-G4</f>
         <v/>
       </c>
       <c r="I4" s="8" t="n">
-        <v>0.3672726154327393</v>
+        <v>0.2000606060028076</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>220.7056279460589</v>
+        <v>195.6758897503217</v>
       </c>
     </row>
     <row r="5">
@@ -3881,250 +4207,158 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>p015</t>
+          <t>c03</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>p015</t>
+          <t>c03</t>
         </is>
       </c>
       <c r="D5" s="10" t="n">
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>9.879232901906896</v>
+        <v>12.64454874803373</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.619753613356174</v>
+        <v>12.49638755346465</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>10.07038371983996</v>
+        <v>11.45864820877159</v>
       </c>
       <c r="H5" s="3">
         <f>E5-G5</f>
         <v/>
       </c>
       <c r="I5" s="8" t="n">
-        <v>0.2159069329500198</v>
+        <v>0.1795676499605179</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>186.3760811726252</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+        <v>195.8286578893662</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Averages per setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Attacks</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>S1 no teacher (CE only)</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>p021</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>p021</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>10.15026036519444</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>9.839114019807274</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>9.450420919396539</v>
-      </c>
-      <c r="H6" s="3">
-        <f>E6-G6</f>
-        <v/>
-      </c>
-      <c r="I6" s="8" t="n">
-        <v>0.5500203967094421</v>
-      </c>
-      <c r="J6" s="9" t="n">
-        <v>201.278364944458</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>p035</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>p035</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>9.769899243281543</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>9.753765040360975</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>9.082354949847025</v>
-      </c>
-      <c r="H7" s="3">
-        <f>E7-G7</f>
-        <v/>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>0.1388921737670898</v>
-      </c>
-      <c r="J7" s="9" t="n">
-        <v>203.8180212457975</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Averages per setting</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>Attacks</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>Label restoration acc</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>PSNR consensus (dB)</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>PSNR best seed (dB)</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>PSNR gray floor (dB)</t>
-        </is>
-      </c>
-      <c r="G10" s="1" t="inlineStr">
-        <is>
-          <t>Consensus - floor (dB)</t>
-        </is>
+      <c r="B9">
+        <f>COUNTIF(A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="10">
+        <f>AVERAGEIFS(D$2:D$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="3">
+        <f>AVERAGEIFS(E$2:E$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="E9" s="3">
+        <f>AVERAGEIFS(F$2:F$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="3">
+        <f>AVERAGEIFS(G$2:G$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="3">
+        <f>AVERAGEIFS(H$2:H$5,A$2:A$5,A9)</f>
+        <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only)</t>
-        </is>
-      </c>
-      <c r="B11">
-        <f>COUNTIF(A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="C11" s="10">
-        <f>AVERAGEIFS(D$2:D$7,A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="D11" s="3">
-        <f>AVERAGEIFS(E$2:E$7,A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="E11" s="3">
-        <f>AVERAGEIFS(F$2:F$7,A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="F11" s="3">
-        <f>AVERAGEIFS(G$2:G$7,A$2:A$7,A11)</f>
-        <v/>
-      </c>
-      <c r="G11" s="3">
-        <f>AVERAGEIFS(H$2:H$7,A$2:A$7,A11)</f>
-        <v/>
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Threat model: honest-but-curious server sees one client's student gradient for one local step (batch 8, distinct labels, round-30 global student). Private teacher and projector are unknown to the attacker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>PSNR: images in [0,1], reconstructions matched one-to-one to ground truth (Hungarian), averaged over the batch. Consensus = pixel mean over seeds; best seed = lowest gradient-matching loss (attacker-selectable).</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Threat model: honest-but-curious server sees one client's student gradient for one local step (batch 8, distinct labels, round-30 global student). Private teacher and projector are unknown to the attacker.</t>
+          <t>Gray floor: PSNR of a uniform gray image; a reconstruction below it carries no recoverable pixel information.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>PSNR: images in [0,1], reconstructions matched one-to-one to ground truth (Hungarian), averaged over the batch. Consensus = pixel mean over seeds; best seed = lowest gradient-matching loss (attacker-selectable).</t>
+          <t>Run c00: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Gray floor: PSNR of a uniform gray image; a reconstruction below it carries no recoverable pixel information.</t>
+          <t>Run c01: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Run p002: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+          <t>Run c02: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Run p012: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Run p014: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Run p015: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Run p021: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Run p035: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+          <t>Run c03: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A123"/>
+  <dimension ref="A1:A75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4152,42 +4386,28 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>S1 no teacher (CE only) - client p002 - run p002</t>
+          <t>S1 no teacher (CE only) - client c00 - run c00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>S1 no teacher (CE only) - client p012 - run p012</t>
+          <t>S1 no teacher (CE only) - client c01 - run c01</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>S1 no teacher (CE only) - client p014 - run p014</t>
+          <t>S1 no teacher (CE only) - client c02 - run c02</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>S1 no teacher (CE only) - client p015 - run p015</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p021 - run p021</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="4" t="inlineStr">
-        <is>
-          <t>S1 no teacher (CE only) - client p035 - run p035</t>
+          <t>S1 no teacher (CE only) - client c03 - run c03</t>
         </is>
       </c>
     </row>
@@ -4198,6 +4418,414 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Run (config folder)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Final grad-match loss (best seed)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Time (min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>c00</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>c00</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>13.57195560883181</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>13.64638531978712</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>12.34300487756501</v>
+      </c>
+      <c r="H2" s="3">
+        <f>E2-G2</f>
+        <v/>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>0.09540053457021713</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>392.5580261826515</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>c01</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>c01</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>13.5697719779718</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>13.94416378795383</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>10.39194379566542</v>
+      </c>
+      <c r="H3" s="3">
+        <f>E3-G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>0.1208854019641876</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>396.4476766308149</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>c02</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>c02</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>15.77217324848811</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>15.38531934326772</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>12.68074810257826</v>
+      </c>
+      <c r="H4" s="3">
+        <f>E4-G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>0.1262353658676147</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>363.5754559993744</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>c03</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>c03</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>12.97776222895058</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>13.0901060601308</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>11.45864820877159</v>
+      </c>
+      <c r="H5" s="3">
+        <f>E5-G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.11110969632864</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>368.3977769295374</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Averages per setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Attacks</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>COUNTIF(A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="10">
+        <f>AVERAGEIFS(D$2:D$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="3">
+        <f>AVERAGEIFS(E$2:E$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="E9" s="3">
+        <f>AVERAGEIFS(F$2:F$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="3">
+        <f>AVERAGEIFS(G$2:G$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="3">
+        <f>AVERAGEIFS(H$2:H$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Threat model: honest-but-curious server sees one client's student gradient for one local step (batch 8, distinct labels, round-30 global student). Private teacher and projector are unknown to the attacker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>PSNR: images in [0,1], reconstructions matched one-to-one to ground truth (Hungarian), averaged over the batch. Consensus = pixel mean over seeds; best seed = lowest gradient-matching loss (attacker-selectable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Gray floor: PSNR of a uniform gray image; a reconstruction below it carries no recoverable pixel information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Run c00: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Run c01: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Run c02: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Run c03: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Each grid: row 1 = actual batch, row 2 = consensus reconstruction, row 3 = best-seed reconstruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client c00 - run c00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client c01 - run c01</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client c02 - run c02</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client c03 - run c03</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4273,7 +4901,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -4290,10 +4918,10 @@
         <v>0.75</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>11.95569679194365</v>
+        <v>10.18981834941837</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>11.9642847229547</v>
+        <v>10.02273675431274</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>9.40250867502931</v>
@@ -4303,16 +4931,16 @@
         <v/>
       </c>
       <c r="I2" s="8" t="n">
-        <v>0.03264361619949341</v>
+        <v>0.1020715609192848</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>380.7995753804843</v>
+        <v>202.1691537022591</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -4329,10 +4957,10 @@
         <v>0.875</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>12.01081569052551</v>
+        <v>10.92384761775596</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>11.82164962106386</v>
+        <v>10.76693620718362</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>9.988775402453584</v>
@@ -4342,16 +4970,16 @@
         <v/>
       </c>
       <c r="I3" s="8" t="n">
-        <v>0.03365790098905563</v>
+        <v>0.08336395770311356</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>388.8103427012762</v>
+        <v>206.3601462403933</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -4368,10 +4996,10 @@
         <v>0.75</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>10.47159694146267</v>
+        <v>10.65960550177276</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>10.33662003823281</v>
+        <v>10.35919985618149</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>10.14880432187795</v>
@@ -4381,16 +5009,16 @@
         <v/>
       </c>
       <c r="I4" s="8" t="n">
-        <v>0.03335896506905556</v>
+        <v>0.3672726154327393</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>417.1127759496371</v>
+        <v>220.7056279460589</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -4407,10 +5035,10 @@
         <v>0.75</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>12.00279410983525</v>
+        <v>9.879232901906896</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>11.54788435056746</v>
+        <v>9.619753613356174</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>10.07038371983996</v>
@@ -4420,16 +5048,16 @@
         <v/>
       </c>
       <c r="I5" s="8" t="n">
-        <v>0.02070866525173187</v>
+        <v>0.2159069329500198</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>341.1732741475105</v>
+        <v>186.3760811726252</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -4446,10 +5074,10 @@
         <v>0.75</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>10.27059412332502</v>
+        <v>10.15026036519444</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10.04729325639967</v>
+        <v>9.839114019807274</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>9.450420919396539</v>
@@ -4459,16 +5087,16 @@
         <v/>
       </c>
       <c r="I6" s="8" t="n">
-        <v>0.03082906268537045</v>
+        <v>0.5500203967094421</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>377.3576625108719</v>
+        <v>201.278364944458</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -4485,10 +5113,10 @@
         <v>0.75</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>9.597271589453804</v>
+        <v>9.769899243281543</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>9.647701764458878</v>
+        <v>9.753765040360975</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>9.082354949847025</v>
@@ -4498,10 +5126,10 @@
         <v/>
       </c>
       <c r="I7" s="8" t="n">
-        <v>0.01635104231536388</v>
+        <v>0.1388921737670898</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>384.069699660937</v>
+        <v>203.8180212457975</v>
       </c>
     </row>
     <row r="9">
@@ -4551,7 +5179,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+          <t>S1 no teacher (CE only)</t>
         </is>
       </c>
       <c r="B11">
@@ -4644,99 +5272,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A123"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Each grid: row 1 = actual batch, row 2 = consensus reconstruction, row 3 = best-seed reconstruction</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p002 - run p002</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p012 - run p012</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p014 - run p014</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p015 - run p015</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="4" t="inlineStr">
-        <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p021 - run p021</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="4" t="inlineStr">
-        <is>
-          <t>S2 DINOv2 ViT-B/14 surrogate - client p035 - run p035</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>psnr_gain_all_clients.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>psnr_gain_vs_iteration.png</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5491,6 +6026,671 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A123"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Each grid: row 1 = actual batch, row 2 = consensus reconstruction, row 3 = best-seed reconstruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p002 - run p002</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p012 - run p012</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p014 - run p014</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p015 - run p015</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p021 - run p021</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p035 - run p035</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Run (config folder)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Final grad-match loss (best seed)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Time (min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>p002</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>p002</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>11.95569679194365</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>11.9642847229547</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>9.40250867502931</v>
+      </c>
+      <c r="H2" s="3">
+        <f>E2-G2</f>
+        <v/>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>0.03264361619949341</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>380.7995753804843</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>12.01081569052551</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>11.82164962106386</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>9.988775402453584</v>
+      </c>
+      <c r="H3" s="3">
+        <f>E3-G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>0.03365790098905563</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>388.8103427012762</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>10.47159694146267</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>10.33662003823281</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>10.14880432187795</v>
+      </c>
+      <c r="H4" s="3">
+        <f>E4-G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>0.03335896506905556</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>417.1127759496371</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>12.00279410983525</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>11.54788435056746</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>10.07038371983996</v>
+      </c>
+      <c r="H5" s="3">
+        <f>E5-G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.02070866525173187</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>341.1732741475105</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>p021</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>p021</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>10.27059412332502</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>10.04729325639967</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>9.450420919396539</v>
+      </c>
+      <c r="H6" s="3">
+        <f>E6-G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>0.03082906268537045</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>377.3576625108719</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>9.597271589453804</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>9.647701764458878</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>9.082354949847025</v>
+      </c>
+      <c r="H7" s="3">
+        <f>E7-G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>0.01635104231536388</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>384.069699660937</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Averages per setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Attacks</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>COUNTIF(A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="10">
+        <f>AVERAGEIFS(D$2:D$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="3">
+        <f>AVERAGEIFS(E$2:E$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="E11" s="3">
+        <f>AVERAGEIFS(F$2:F$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="3">
+        <f>AVERAGEIFS(G$2:G$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="3">
+        <f>AVERAGEIFS(H$2:H$7,A$2:A$7,A11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Threat model: honest-but-curious server sees one client's student gradient for one local step (batch 8, distinct labels, round-30 global student). Private teacher and projector are unknown to the attacker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>PSNR: images in [0,1], reconstructions matched one-to-one to ground truth (Hungarian), averaged over the batch. Consensus = pixel mean over seeds; best seed = lowest gradient-matching loss (attacker-selectable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Gray floor: PSNR of a uniform gray image; a reconstruction below it carries no recoverable pixel information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Run p002: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Run p012: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Run p014: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Run p015: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Run p021: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Run p035: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A123"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Each grid: row 1 = actual batch, row 2 = consensus reconstruction, row 3 = best-seed reconstruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p002 - run p002</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p012 - run p012</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p014 - run p014</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p015 - run p015</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p021 - run p021</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p035 - run p035</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_all_clients.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_vs_iteration.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_all_clients.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_vs_iteration.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_all_clients.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_vs_iteration.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add State Farm frozen-teacher GradInversion results (S1, S2, 20k; p012, p014, p015, p035)
</commit_message>
<xml_diff>
--- a/fedkd_gia/results/fedkd_gia_results.xlsx
+++ b/fedkd_gia/results/fedkd_gia_results.xlsx
@@ -33,10 +33,16 @@
     <sheet name="S1_full_Images" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="S2_full" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="S2_full_Images" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="CIFAR_v3_S1_full_Plots" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="CIFAR_v3_S2_full_Plots" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="S1_full_Plots" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="S2_full_Plots" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="SF_frozen_S1_full" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="SF_frozen_S1_full_Images" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="SF_frozen_S2_full" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="SF_frozen_S2_full_Images" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="CIFAR_v3_S1_full_Plots" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="CIFAR_v3_S2_full_Plots" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="S1_full_Plots" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="S2_full_Plots" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="SF_frozen_S1_full_Plots" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="SF_frozen_S2_full_Plots" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -277,6 +283,171 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4819650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4276725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4819650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4276725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4819650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4276725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -711,10 +882,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>1</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="4819650"/>
+    <ext cx="10477500" cy="3924300"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -736,10 +907,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>30</row>
+      <row>27</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="4276725"/>
+    <ext cx="10477500" cy="3924300"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -747,6 +918,56 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>75</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -766,10 +987,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>1</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="4819650"/>
+    <ext cx="10477500" cy="3924300"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -791,10 +1012,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>30</row>
+      <row>27</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="4276725"/>
+    <ext cx="10477500" cy="3924300"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -802,6 +1023,56 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>75</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="3924300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -871,6 +1142,61 @@
 </file>
 
 <file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4819650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="4276725"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -8982,26 +9308,355 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>psnr_gain_all_clients.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>psnr_gain_vs_iteration.png</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Run (config folder)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Final grad-match loss (best seed)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Time (min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>12.41782966737943</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>12.05173305143371</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>10.02816686747077</v>
+      </c>
+      <c r="H2" s="3">
+        <f>E2-G2</f>
+        <v/>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>0.07908179610967636</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>199.4315705100695</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>11.76308969645838</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>11.67965256627977</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>10.07950395309883</v>
+      </c>
+      <c r="H3" s="3">
+        <f>E3-G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>0.0659596174955368</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>228.6125053405762</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>12.5823567408111</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>12.31515529311671</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>9.913487438257205</v>
+      </c>
+      <c r="H4" s="3">
+        <f>E4-G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>0.08273918926715851</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>228.5407834927241</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>10.44054239390326</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>10.00884598059407</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>9.145437989527831</v>
+      </c>
+      <c r="H5" s="3">
+        <f>E5-G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.1659089624881744</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>202.1758806387583</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Averages per setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Attacks</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only)</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>COUNTIF(A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="10">
+        <f>AVERAGEIFS(D$2:D$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="3">
+        <f>AVERAGEIFS(E$2:E$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="E9" s="3">
+        <f>AVERAGEIFS(F$2:F$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="3">
+        <f>AVERAGEIFS(G$2:G$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="3">
+        <f>AVERAGEIFS(H$2:H$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Threat model: honest-but-curious server sees one client's student gradient for one local step (batch 8, distinct labels, round-30 global student). Private teacher and projector are unknown to the attacker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>PSNR: images in [0,1], reconstructions matched one-to-one to ground truth (Hungarian), averaged over the batch. Consensus = pixel mean over seeds; best seed = lowest gradient-matching loss (attacker-selectable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Gray floor: PSNR of a uniform gray image; a reconstruction below it carries no recoverable pixel information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Run p012: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Run p014: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Run p015: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Run p035: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -9011,20 +9666,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>psnr_gain_all_clients.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>psnr_gain_vs_iteration.png</t>
+          <t>Each grid: row 1 = actual batch, row 2 = consensus reconstruction, row 3 = best-seed reconstruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p012 - run p012</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p014 - run p014</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p015 - run p015</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>S1 no teacher (CE only) - client p035 - run p035</t>
         </is>
       </c>
     </row>
@@ -9040,26 +9716,355 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>psnr_gain_all_clients.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>psnr_gain_vs_iteration.png</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Run (config folder)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Final grad-match loss (best seed)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Time (min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>p012</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>13.19801240812795</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>12.8158548821955</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>10.02816686747077</v>
+      </c>
+      <c r="H2" s="3">
+        <f>E2-G2</f>
+        <v/>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>0.03566859662532806</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>375.1349317948024</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>p014</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>12.07076485970101</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>11.83967941280906</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>10.07950395309883</v>
+      </c>
+      <c r="H3" s="3">
+        <f>E3-G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>0.02988815866410732</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>429.0620844841004</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>p015</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>12.84320071111081</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>12.53121800586938</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>9.913487438257205</v>
+      </c>
+      <c r="H4" s="3">
+        <f>E4-G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>0.02659221366047859</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>429.8819097320239</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>p035</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>10.94220920275331</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>10.34322911185853</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>9.145437989527831</v>
+      </c>
+      <c r="H5" s="3">
+        <f>E5-G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.0642721951007843</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>379.8180241823196</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Averages per setting</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Attacks</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Label restoration acc</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>PSNR consensus (dB)</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>PSNR best seed (dB)</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>PSNR gray floor (dB)</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Consensus - floor (dB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>COUNTIF(A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="10">
+        <f>AVERAGEIFS(D$2:D$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="3">
+        <f>AVERAGEIFS(E$2:E$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="E9" s="3">
+        <f>AVERAGEIFS(F$2:F$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="3">
+        <f>AVERAGEIFS(G$2:G$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="3">
+        <f>AVERAGEIFS(H$2:H$5,A$2:A$5,A9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Threat model: honest-but-curious server sees one client's student gradient for one local step (batch 8, distinct labels, round-30 global student). Private teacher and projector are unknown to the attacker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>PSNR: images in [0,1], reconstructions matched one-to-one to ground truth (Hungarian), averaged over the batch. Consensus = pixel mean over seeds; best seed = lowest gradient-matching loss (attacker-selectable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Gray floor: PSNR of a uniform gray image; a reconstruction below it carries no recoverable pixel information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Run p012: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Run p014: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Run p015: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Run p035: {"iterations": 20000, "num_seeds": 2, "lr": 0.1, "alpha_tv": 1.0, "alpha_l2": 1e-06, "alpha_group": 0.01, "alpha_noise": 0.0}</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -9559,6 +10564,201 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Each grid: row 1 = actual batch, row 2 = consensus reconstruction, row 3 = best-seed reconstruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p012 - run p012</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p014 - run p014</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p015 - run p015</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>S2 DINOv2 ViT-B/14 surrogate - client p035 - run p035</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_all_clients.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_vs_iteration.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_all_clients.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_vs_iteration.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_all_clients.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_vs_iteration.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_all_clients.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_vs_iteration.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_all_clients.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>psnr_gain_vs_iteration.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>